<commit_message>
Updated excel file with subset of molecules
</commit_message>
<xml_diff>
--- a/predicted_ee.xlsx
+++ b/predicted_ee.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zhuan08/Programming Projects/oled-project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83341DD5-415B-6B45-AF3C-89178954DE73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B175FE19-D00A-094D-A065-728382624BED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="680" yWindow="740" windowWidth="28040" windowHeight="16840" xr2:uid="{2FDB0681-3AEB-6747-B8EB-32CB84415B37}"/>
+    <workbookView xWindow="680" yWindow="740" windowWidth="28040" windowHeight="16840" activeTab="1" xr2:uid="{2FDB0681-3AEB-6747-B8EB-32CB84415B37}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Fullset" sheetId="1" r:id="rId1"/>
+    <sheet name="Subset" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="79">
   <si>
     <t>mol_id</t>
   </si>
@@ -279,7 +280,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -299,13 +300,44 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF006100"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF9C0006"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -320,9 +352,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -700,7 +735,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{8EB59CE3-52B1-9E40-AF10-FB849D638F2E}" type="CELLRANGE">
+                    <a:fld id="{4D16461C-B40A-214C-B35C-16E883AAEAF5}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -738,7 +773,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{A57AC2A3-F392-CE48-8484-6F8A200FD93F}" type="CELLRANGE">
+                    <a:fld id="{12363CAC-E3EE-5A49-A116-A2E6C85A5613}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -776,7 +811,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{BEBB19F0-5E37-644E-BDAE-391FE3E4C702}" type="CELLRANGE">
+                    <a:fld id="{E4B25AE9-678A-8240-B594-F3DE8FD4FD77}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -814,7 +849,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{92FA9EB4-7E61-1E43-9231-CEC8B35AF23D}" type="CELLRANGE">
+                    <a:fld id="{37057BB2-B867-4047-A168-19BBAE199F92}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -900,7 +935,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{BC9D1E6A-4E83-3B4A-BE95-D6FFECCA5F5D}" type="CELLRANGE">
+                    <a:fld id="{74712E31-9678-D740-BB78-AE1591231F2B}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1257,7 +1292,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{8FFF0E5F-8AA4-0545-8DC5-D716B3C1B669}" type="CELLRANGE">
+                    <a:fld id="{B1D9F75B-75D6-284A-AAF8-526A41250654}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1404,7 +1439,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{D5A617CE-3DE9-7945-8E08-1F3651958E63}" type="CELLRANGE">
+                    <a:fld id="{B1B865BB-3539-5A48-BA33-F9AC7B124AC8}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1442,7 +1477,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{2C148650-008A-1F4B-9C21-1C50E98E3849}" type="CELLRANGE">
+                    <a:fld id="{252F5563-F08E-6642-90B1-0A9C3423DEAA}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1669,7 +1704,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{BBC4E310-B9A2-E64C-9A5C-DD36FFD8E806}" type="CELLRANGE">
+                    <a:fld id="{23B6A2D3-A0A6-6741-9A01-6C30CEFBCBA9}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1734,7 +1769,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{AA09DABA-8B94-2544-A253-79B6F645A9AF}" type="CELLRANGE">
+                    <a:fld id="{67F5326D-7968-BC4E-92FE-7E14EAE6D860}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1799,7 +1834,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{7A116439-C037-A445-AB9A-0B8893E7FE73}" type="CELLRANGE">
+                    <a:fld id="{4319781B-9879-4E4F-BA93-63BE385E56FF}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1972,7 +2007,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{3848A206-F9F7-5044-BDF5-7D08414142C3}" type="CELLRANGE">
+                    <a:fld id="{722DCA5B-51A5-CF45-81C8-47B8B4DFCD15}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2010,7 +2045,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{2687AE00-F309-244D-8A70-C788A652E498}" type="CELLRANGE">
+                    <a:fld id="{D2AE9628-3E18-7346-A36E-E13A614116B4}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2048,7 +2083,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{EF14E922-1F41-BC42-94B5-2E7778FB396D}" type="CELLRANGE">
+                    <a:fld id="{1F6D1D2E-F787-3E4B-A86C-8DF17BD183BE}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2086,7 +2121,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{D4C3BC00-9B8E-AA4F-874B-B3438CBA6A94}" type="CELLRANGE">
+                    <a:fld id="{9CA52215-6816-6A4C-944F-A9B3A07F6291}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2145,7 +2180,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{3E1EBB86-1ACA-2C4B-BBCB-44653BA3F9A0}" type="CELLRANGE">
+                    <a:fld id="{D46B6908-C8F4-9F48-849E-17E8ABD13374}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2178,7 +2213,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{D8B2C93B-6D39-F242-9151-B56183008C8B}" type="CELLRANGE">
+                    <a:fld id="{4C49D0CB-A002-354D-BED1-8C597C5638D3}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2211,7 +2246,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{C58F3C15-0541-6B42-8F1C-27A31DC614F6}" type="CELLRANGE">
+                    <a:fld id="{7F80CA86-F066-AF49-B3BE-95A02ADC00B5}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2250,7 +2285,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{35A271FB-4380-824A-B020-2CF9E50B61CE}" type="CELLRANGE">
+                    <a:fld id="{3D33CAE0-5C93-AE46-8366-64708EFA8AE3}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2288,7 +2323,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{B3250B32-073A-744A-AC5A-C6EB156249A2}" type="CELLRANGE">
+                    <a:fld id="{20991813-12E1-C64C-9BD8-46EFB810C8B1}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2326,7 +2361,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{065CA9FA-9328-594F-B67B-E557822604BB}" type="CELLRANGE">
+                    <a:fld id="{FDCE9B32-7E83-754C-8C9B-7AC98572FFD5}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2364,7 +2399,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{EECD72A9-254F-B54A-AE2E-2FBA1022E25A}" type="CELLRANGE">
+                    <a:fld id="{04BD476B-08F8-BB48-89EE-5E9D1EBC7506}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2402,7 +2437,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{8B527580-93B5-E745-923A-D9270363C9C5}" type="CELLRANGE">
+                    <a:fld id="{82F2FBF2-5802-1A48-BF0D-8F2D59BC5460}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2434,7 +2469,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{545B9B7A-032F-F54D-8035-5444105302F4}" type="CELLRANGE">
+                    <a:fld id="{D3B5B546-DEBD-BE4D-83EF-EDC4E4027F29}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2473,7 +2508,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{C89E2F26-7D4A-E94A-91D8-9FC89061CB26}" type="CELLRANGE">
+                    <a:fld id="{391855A8-DA2E-904F-83C3-D81698EE1FA5}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2511,7 +2546,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{FE69D1AA-163E-CF4D-892A-A4703BDD5C64}" type="CELLRANGE">
+                    <a:fld id="{1A183D5E-C8B5-2C4B-B06F-09FD0B04ABFF}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2549,7 +2584,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{E122E697-67C3-9D4F-82E0-E33E4D82B43E}" type="CELLRANGE">
+                    <a:fld id="{DF2CF14C-8923-374C-8649-36D4B60E7190}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2581,7 +2616,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{3B9A5B5C-D3B4-244A-94F5-F4339336AA5B}" type="CELLRANGE">
+                    <a:fld id="{F37BCDB8-DEDA-6B47-9173-CCB2186051C6}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2620,7 +2655,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{FEF9AAC5-1612-A04C-B113-6785C7A29DC0}" type="CELLRANGE">
+                    <a:fld id="{1DF6FC84-DC8D-3941-A725-9060A5C1A624}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2658,7 +2693,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{474494A4-9403-3D45-B11D-CA8E08F0FB29}" type="CELLRANGE">
+                    <a:fld id="{1AA57511-7804-0240-B82C-FE3213882D0B}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2696,7 +2731,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{6AB63A4F-A5AE-2F47-ACAB-FF74494E4179}" type="CELLRANGE">
+                    <a:fld id="{20910B88-20E3-D34E-A65E-420D5DAE8F85}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2734,7 +2769,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{059A7467-D3FA-2B4F-86A2-5F93095A2D4B}" type="CELLRANGE">
+                    <a:fld id="{477BE4FC-BCC4-E64B-9531-DAF78C857B22}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2870,7 +2905,7 @@
           </c:trendline>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet1!$C$2:$C$74</c:f>
+              <c:f>Fullset!$C$2:$C$74</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="73"/>
@@ -3098,7 +3133,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$B$2:$B$74</c:f>
+              <c:f>Fullset!$B$2:$B$74</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="73"/>
@@ -3205,7 +3240,7 @@
           <c:extLst>
             <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
               <c15:datalabelsRange>
-                <c15:f>Sheet1!$A$2:$A$74</c15:f>
+                <c15:f>Fullset!$A$2:$A$74</c15:f>
                 <c15:dlblRangeCache>
                   <c:ptCount val="73"/>
                   <c:pt idx="0">
@@ -3710,7 +3745,968 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Correlation</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" baseline="0"/>
+              <a:t> Graph</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln w="38100" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:dLbl>
+              <c:idx val="0"/>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{371F8D2E-2E66-AB46-AF92-DDEFDE6A5791}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[CELLRANGE]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="en-US"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000005-DD04-5241-B7E1-B5421D1EBE01}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="1"/>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{D470ADE2-F4E9-B34B-B5EC-B719AD52D991}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[CELLRANGE]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="en-US"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000006-DD04-5241-B7E1-B5421D1EBE01}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="2"/>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{441096B5-957E-2747-9207-941199611E0D}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[CELLRANGE]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="en-US"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000007-DD04-5241-B7E1-B5421D1EBE01}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="3"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-0.13888888888888898"/>
+                  <c:y val="6.4814814814814728E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{37BF8727-0BB9-284A-8828-323A8DFD01E7}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[CELLRANGE]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="en-US"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000004-DD04-5241-B7E1-B5421D1EBE01}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="4"/>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{682AB4C6-B89D-104C-8EC1-C17E53826B05}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[CELLRANGE]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="en-US"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000008-DD04-5241-B7E1-B5421D1EBE01}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="5"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-3.3333333333333437E-2"/>
+                  <c:y val="-8.7962962962963048E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{9C8A5AFA-190E-7942-B839-1F30AF9AF053}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[CELLRANGE]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="en-US"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000003-DD04-5241-B7E1-B5421D1EBE01}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="6"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="2.7777777777777776E-2"/>
+                  <c:y val="-4.1666666666666755E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{8876A23B-EABE-E64E-B89A-2F1C1D1E8602}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[CELLRANGE]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="en-US"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000002-DD04-5241-B7E1-B5421D1EBE01}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="7"/>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{032D4673-DAA3-0C45-8C74-C6A9193829E9}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[CELLRANGE]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="en-US"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000009-DD04-5241-B7E1-B5421D1EBE01}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="8"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-1.3888888888888888E-2"/>
+                  <c:y val="-6.0185185185185355E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{02C85974-1B21-6146-8903-4F8E989481FB}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[CELLRANGE]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="en-US"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{0000000A-DD04-5241-B7E1-B5421D1EBE01}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:spPr>
+              <a:solidFill>
+                <a:sysClr val="window" lastClr="FFFFFF"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000">
+                    <a:lumMod val="25000"/>
+                    <a:lumOff val="75000"/>
+                  </a:sysClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="dk1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:spPr xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                  <a:prstGeom prst="wedgeRectCallout">
+                    <a:avLst/>
+                  </a:prstGeom>
+                  <a:noFill/>
+                  <a:ln>
+                    <a:noFill/>
+                  </a:ln>
+                </c15:spPr>
+                <c15:showDataLabelsRange val="1"/>
+                <c15:showLeaderLines val="0"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="1"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="0.12489457567804024"/>
+                  <c:y val="-0.50395596383785357"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Subset!$B$2:$B$10</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>2.8054299999999999</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2.2878229999999999</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2.3134329999999999</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2.6050420000000001</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2.5726140000000002</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2.627119</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2.6956519999999999</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>2.4409450000000001</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>2.655246</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Subset!$C$2:$C$10</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>0.179053136</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2.024669158</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.98336665700000003</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.51631367399999994</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2.2009162440000001</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.80487891099999997</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.80487913499999997</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>2.14302729</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>9.0716412999999996E-2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+              <c15:datalabelsRange>
+                <c15:f>Subset!$A$2:$A$10</c15:f>
+                <c15:dlblRangeCache>
+                  <c:ptCount val="9"/>
+                  <c:pt idx="0">
+                    <c:v>QAYZZ04</c:v>
+                  </c:pt>
+                  <c:pt idx="1">
+                    <c:v>LOKZZ01</c:v>
+                  </c:pt>
+                  <c:pt idx="2">
+                    <c:v>UVEFAE</c:v>
+                  </c:pt>
+                  <c:pt idx="3">
+                    <c:v>CUYZZ03</c:v>
+                  </c:pt>
+                  <c:pt idx="4">
+                    <c:v>CUYRAS</c:v>
+                  </c:pt>
+                  <c:pt idx="5">
+                    <c:v>CUYZZ07</c:v>
+                  </c:pt>
+                  <c:pt idx="6">
+                    <c:v>CUYZZ08</c:v>
+                  </c:pt>
+                  <c:pt idx="7">
+                    <c:v>CUYZZ09</c:v>
+                  </c:pt>
+                  <c:pt idx="8">
+                    <c:v>IJUZZ04</c:v>
+                  </c:pt>
+                </c15:dlblRangeCache>
+              </c15:datalabelsRange>
+            </c:ext>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-DD04-5241-B7E1-B5421D1EBE01}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="774092640"/>
+        <c:axId val="774063056"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="774092640"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:min val="2.2000000000000002"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Actual EE</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="774063056"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="774063056"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Predicted</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" baseline="0"/>
+                  <a:t> EE</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="774092640"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -4266,20 +5262,536 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>474767</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>130560</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>652567</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>105160</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>154299</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>71215</xdr:rowOff>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>332099</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>45815</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -4287,6 +5799,47 @@
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0EA83122-1990-BFEF-763B-804789A6106C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>110314</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>83802</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>557132</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>175761</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="4" name="Chart 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{86D8DF25-4F7A-D6DE-2103-96EAF2D0BA11}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -5405,4 +6958,125 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD3992E0-094E-8A42-B323-007503EE2A7D}">
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" s="3">
+        <v>2.8054299999999999</v>
+      </c>
+      <c r="C2" s="3">
+        <v>0.179053136</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" s="4">
+        <v>2.2878229999999999</v>
+      </c>
+      <c r="C3" s="4">
+        <v>2.024669158</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B4" s="3">
+        <v>2.3134329999999999</v>
+      </c>
+      <c r="C4" s="3">
+        <v>0.98336665700000003</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B5" s="3">
+        <v>2.6050420000000001</v>
+      </c>
+      <c r="C5" s="3">
+        <v>0.51631367399999994</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6" s="4">
+        <v>2.5726140000000002</v>
+      </c>
+      <c r="C6" s="4">
+        <v>2.2009162440000001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B7" s="3">
+        <v>2.627119</v>
+      </c>
+      <c r="C7" s="3">
+        <v>0.80487891099999997</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B8" s="3">
+        <v>2.6956519999999999</v>
+      </c>
+      <c r="C8" s="3">
+        <v>0.80487913499999997</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B9" s="4">
+        <v>2.4409450000000001</v>
+      </c>
+      <c r="C9" s="4">
+        <v>2.14302729</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B10" s="3">
+        <v>2.655246</v>
+      </c>
+      <c r="C10" s="3">
+        <v>9.0716412999999996E-2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Updated singlet_triplet_gap script and predicted_ee excel file
</commit_message>
<xml_diff>
--- a/predicted_ee.xlsx
+++ b/predicted_ee.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zhuan08/Programming Projects/oled-project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7720E833-0009-9849-84A7-698A68B730E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{764CA33E-8E3A-1C4F-9EE1-0AC3F7E6026A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="680" yWindow="740" windowWidth="28040" windowHeight="16840" activeTab="1" xr2:uid="{2FDB0681-3AEB-6747-B8EB-32CB84415B37}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="76">
   <si>
     <t>mol_id</t>
   </si>
@@ -264,16 +264,7 @@
     <t>actual</t>
   </si>
   <si>
-    <t>MIN</t>
-  </si>
-  <si>
-    <t>MAX</t>
-  </si>
-  <si>
-    <t>pred.</t>
-  </si>
-  <si>
-    <t>act.</t>
+    <t>error message</t>
   </si>
 </sst>
 </file>
@@ -735,7 +726,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{9F7F87A3-FC22-9048-8598-50A67A6E7D9B}" type="CELLRANGE">
+                    <a:fld id="{671E256A-F094-2A47-9771-229EB288F3B8}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -773,7 +764,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{5A9DABBF-938A-2742-AC00-24A6FC9A2E1D}" type="CELLRANGE">
+                    <a:fld id="{2049F7BE-5F38-9A4B-895D-31A53476CF4D}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -811,7 +802,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{E85314A8-5023-CE4A-981C-AAE2ED117FB5}" type="CELLRANGE">
+                    <a:fld id="{9C50B368-677F-0342-A924-9328B0932E87}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -849,7 +840,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{92B5F2F6-A8A5-0D44-A70C-E3A36D48E8D5}" type="CELLRANGE">
+                    <a:fld id="{A9F16355-48FE-5347-BB62-2DDC61B556F8}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -935,7 +926,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{4F7541E0-A3EF-144F-BA78-0B7736CE02C4}" type="CELLRANGE">
+                    <a:fld id="{15D1427E-FBD7-5344-A96C-7FCE48C2C21D}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1292,7 +1283,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{C7111205-0DE5-6041-A5B5-547F0F80D888}" type="CELLRANGE">
+                    <a:fld id="{85900E62-36C8-D44B-853A-1F3BCEDD6771}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1439,7 +1430,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{A80F7C35-3415-C846-8C86-ADE2BADAC680}" type="CELLRANGE">
+                    <a:fld id="{C9DB9298-BF26-8146-82A6-EE202BDF84EA}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1477,7 +1468,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{73EE6C51-3311-104A-8BB1-25F1377F44F1}" type="CELLRANGE">
+                    <a:fld id="{30F2430F-C393-9E4C-9CFE-C15C6AC06B6D}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1704,7 +1695,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{54FDF369-1CDB-4D42-8C6F-9BAD2100AF76}" type="CELLRANGE">
+                    <a:fld id="{1945CC53-7840-C94E-A225-5A193CB81F0C}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1769,7 +1760,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{70F032CC-9EE3-0045-B1ED-C57EEDB42CA9}" type="CELLRANGE">
+                    <a:fld id="{7A7BBFB0-14E8-E34A-9938-AFB48E712359}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1834,7 +1825,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{0DC86397-7AC7-EF43-994E-DB02AE98F01A}" type="CELLRANGE">
+                    <a:fld id="{EF3B390C-CACA-334C-8452-7107118C2863}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2007,7 +1998,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{C9124AB5-9243-914E-9F86-3D61D9CAFDFC}" type="CELLRANGE">
+                    <a:fld id="{F98FE3AC-ACFD-F647-A8DD-E3709DC4FA9A}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2045,7 +2036,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{B07D01DF-0D81-3E41-AC61-52689B6233B6}" type="CELLRANGE">
+                    <a:fld id="{FEB9EF0E-13C8-1C44-9C12-AB4636B51A80}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2083,7 +2074,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{7A03464E-7404-254C-B1C2-0CCB4ED5364C}" type="CELLRANGE">
+                    <a:fld id="{8C293FF3-7361-C142-875C-74E8A7628B0E}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2121,7 +2112,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{FBA7BAA1-15C7-5B4D-B884-F44C7CEFB10E}" type="CELLRANGE">
+                    <a:fld id="{0287557D-7E9D-7B45-9206-1A5E1457A82A}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2180,7 +2171,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{6B3AF1A9-F60B-4F47-8191-98FCBA17F053}" type="CELLRANGE">
+                    <a:fld id="{F69E69A2-2E76-CC4A-871D-098FD4951080}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2213,7 +2204,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{8CC3A46E-BCB1-2B4A-89D5-64FF9A40DB58}" type="CELLRANGE">
+                    <a:fld id="{FAB8CCC1-19BD-A34F-BBD9-8EB973259D73}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2246,7 +2237,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{FD47C7FA-AF1B-E245-8E09-45ECE9A552D9}" type="CELLRANGE">
+                    <a:fld id="{1E8E91D7-1F77-674A-8AB9-E5E84C2A628B}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2285,7 +2276,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{50278100-68A4-C947-A243-7D74B173B95F}" type="CELLRANGE">
+                    <a:fld id="{1EF93158-6AE1-4D4F-A5AF-A59D67C7F96E}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2323,7 +2314,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{45688F99-882A-9347-9AB0-6D5172CFD3A6}" type="CELLRANGE">
+                    <a:fld id="{08DEB95F-0A03-C24D-A7F1-1F3A06AADB78}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2361,7 +2352,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{588F7AE6-7855-BD4D-A402-8C3E958B6BCB}" type="CELLRANGE">
+                    <a:fld id="{30EEAC4A-7C21-0449-A7A6-14BB54188BBD}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2399,7 +2390,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{98FA0CBF-BEB4-1A42-9ABC-46860910340A}" type="CELLRANGE">
+                    <a:fld id="{5FBDCD96-7780-364B-ACE8-13FE5792BBF3}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2437,7 +2428,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{8D18D0ED-75D9-9F4A-8869-821448FD301B}" type="CELLRANGE">
+                    <a:fld id="{80B7E842-366E-6A44-87BE-F3D81840E863}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2469,7 +2460,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{367F07DC-4B1F-9643-B7E5-936BDEF8CF52}" type="CELLRANGE">
+                    <a:fld id="{18CAAA5D-CF07-2B40-932D-00E3823FD53A}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2508,7 +2499,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{0930F8DD-9D9E-5B42-A4D8-7B28243007CE}" type="CELLRANGE">
+                    <a:fld id="{B800F083-7CA6-A142-9E4E-CE5A4FF5A427}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2546,7 +2537,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{A759D2A7-0FC9-2548-9A12-99CD6AC83C78}" type="CELLRANGE">
+                    <a:fld id="{6FE5BED5-E952-9F47-837B-78B6CF89E425}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2584,7 +2575,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{B214CD1D-4C6A-A74A-99FB-9CD48E8A66F6}" type="CELLRANGE">
+                    <a:fld id="{5AA4F5C6-6898-3944-955D-3E8884E897E2}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2616,7 +2607,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{1693FDFD-1E96-5541-91E7-AF4EF003D3CE}" type="CELLRANGE">
+                    <a:fld id="{4D6F9C73-8001-D14A-A056-5B98C177BFA5}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2655,7 +2646,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{C09B45A4-BB5D-EF4B-A830-85DD1306AB77}" type="CELLRANGE">
+                    <a:fld id="{0CA0EF7B-13B4-3443-854C-7EC9A9C65235}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2693,7 +2684,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{CDE7A2A6-D83C-A240-BBB2-2D53D03B6D36}" type="CELLRANGE">
+                    <a:fld id="{CAFC1FC2-B7FC-4E43-A02D-7BCCEF20B005}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2731,7 +2722,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{C5DDDB19-7858-F946-BCD8-AC9045643114}" type="CELLRANGE">
+                    <a:fld id="{B35B0603-3F02-8449-8348-0D960B6D42CE}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2769,7 +2760,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{C8E1D990-4E3A-5B4F-BBFB-78F36D5B27CD}" type="CELLRANGE">
+                    <a:fld id="{9A2E7B67-874B-6042-A7E5-3689B199E793}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -3858,7 +3849,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{234B65A0-1FA0-7847-8518-480726CBABBE}" type="CELLRANGE">
+                    <a:fld id="{FC975DD8-73AD-274B-8A59-DA59A33B28F2}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -3891,7 +3882,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{0D28E59B-D7BE-CE4A-B7F3-EE7AB64AD39F}" type="CELLRANGE">
+                    <a:fld id="{5D82D4D9-7135-2F45-A13F-65AD2B2C537D}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -3924,7 +3915,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{11C0689B-3C79-F845-BBE1-0BF5E5C08387}" type="CELLRANGE">
+                    <a:fld id="{B97D85D5-6707-C840-B35E-5500F95248E2}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -3963,7 +3954,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{68CC6354-F653-7B4D-A9B4-C9810F226BB7}" type="CELLRANGE">
+                    <a:fld id="{C5665415-58EE-B84F-A3B4-7F2646E1E741}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -3995,7 +3986,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{7E924CE5-10CF-8F44-A4B5-8571BCB21B9F}" type="CELLRANGE">
+                    <a:fld id="{4D158764-D98D-FD4C-B89F-564F3433425B}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -4034,7 +4025,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{87323168-7880-1247-929A-72F8B4469E40}" type="CELLRANGE">
+                    <a:fld id="{09E5FCBC-A5BC-D342-BA33-C3881214EEF2}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -4072,7 +4063,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{CC5C8226-CB97-264D-B435-A253B1A57F0D}" type="CELLRANGE">
+                    <a:fld id="{91905E96-31CE-B442-B120-751770AA62A9}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -4104,7 +4095,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{5AF09935-093B-EF48-9FA3-D9D33BA747EC}" type="CELLRANGE">
+                    <a:fld id="{C4A46D10-6039-DF4E-9550-B319FC0987E0}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -4143,7 +4134,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{E11B020E-9D88-8743-BAE3-80052B6DC8B0}" type="CELLRANGE">
+                    <a:fld id="{89012BB3-8AF8-A143-8AF9-9FF40C1FC64A}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -5782,16 +5773,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>17567</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>16260</xdr:rowOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>55667</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>194060</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>522599</xdr:colOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>560699</xdr:colOff>
       <xdr:row>27</xdr:row>
-      <xdr:rowOff>160115</xdr:rowOff>
+      <xdr:rowOff>134715</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -5823,16 +5814,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>17613</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>18911</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>360606</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>65262</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>464431</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>110871</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>807424</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>157221</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -6177,15 +6168,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44EE2A20-8B5A-884B-A28C-9E065EAA06D6}">
-  <dimension ref="A1:G74"/>
+  <dimension ref="A1:F74"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8.83203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.1640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -6195,14 +6187,11 @@
       <c r="C1" t="s">
         <v>74</v>
       </c>
-      <c r="F1" t="s">
+      <c r="D1" t="s">
         <v>75</v>
       </c>
-      <c r="G1" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -6210,19 +6199,10 @@
       <c r="C2">
         <v>2.6552462526766498</v>
       </c>
-      <c r="E2" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="F2" s="1">
-        <f>MIN(B2:B74)</f>
-        <v>0.25836642727244902</v>
-      </c>
-      <c r="G2">
-        <f>MAX(B2:B74)</f>
-        <v>2.2529607499563999</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
@@ -6230,19 +6210,9 @@
       <c r="C3">
         <v>2.6495726495726402</v>
       </c>
-      <c r="E3" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="F3">
-        <f>MIN(C2:C74)</f>
-        <v>2.0361247947454801</v>
-      </c>
-      <c r="G3">
-        <f>MAX(C2:C74)</f>
-        <v>3.2291666666666599</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="E3" s="1"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -6252,7 +6222,7 @@
       </c>
       <c r="D4" s="1"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
@@ -6262,7 +6232,7 @@
       </c>
       <c r="D5" s="1"/>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>5</v>
       </c>
@@ -6272,7 +6242,7 @@
       </c>
       <c r="D6" s="1"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>6</v>
       </c>
@@ -6282,7 +6252,7 @@
       </c>
       <c r="D7" s="1"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>7</v>
       </c>
@@ -6292,7 +6262,7 @@
       </c>
       <c r="D8" s="1"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>8</v>
       </c>
@@ -6302,7 +6272,7 @@
       </c>
       <c r="D9" s="1"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>9</v>
       </c>
@@ -6314,7 +6284,7 @@
       </c>
       <c r="D10" s="1"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -6326,7 +6296,7 @@
       </c>
       <c r="D11" s="1"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>11</v>
       </c>
@@ -6338,7 +6308,7 @@
       </c>
       <c r="D12" s="1"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -6350,7 +6320,7 @@
       </c>
       <c r="D13" s="1"/>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>13</v>
       </c>
@@ -6360,7 +6330,7 @@
       </c>
       <c r="D14" s="1"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>14</v>
       </c>
@@ -6369,7 +6339,7 @@
       </c>
       <c r="D15" s="1"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>15</v>
       </c>

</xml_diff>

<commit_message>
Updated script to display error messages, and updated excel file
</commit_message>
<xml_diff>
--- a/predicted_ee.xlsx
+++ b/predicted_ee.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zhuan08/Programming Projects/oled-project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{764CA33E-8E3A-1C4F-9EE1-0AC3F7E6026A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFF811BA-649E-B348-BD70-F0BD4062DC0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="680" yWindow="740" windowWidth="28040" windowHeight="16840" activeTab="1" xr2:uid="{2FDB0681-3AEB-6747-B8EB-32CB84415B37}"/>
+    <workbookView xWindow="680" yWindow="740" windowWidth="28040" windowHeight="16840" xr2:uid="{2FDB0681-3AEB-6747-B8EB-32CB84415B37}"/>
   </bookViews>
   <sheets>
     <sheet name="Fullset" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="81">
   <si>
     <t>mol_id</t>
   </si>
@@ -264,14 +264,29 @@
     <t>actual</t>
   </si>
   <si>
-    <t>error message</t>
+    <t>error_msg</t>
+  </si>
+  <si>
+    <t>Doesn't match templates</t>
+  </si>
+  <si>
+    <t>Could not embed molecule.</t>
+  </si>
+  <si>
+    <t>No Error Message</t>
+  </si>
+  <si>
+    <t>Doesn't match templates}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Could not embed molecule  </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -310,6 +325,13 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -343,17 +365,119 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="10">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -726,7 +850,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{671E256A-F094-2A47-9771-229EB288F3B8}" type="CELLRANGE">
+                    <a:fld id="{6E43E011-2946-0544-BA47-9EE81BCAB7ED}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -764,7 +888,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{2049F7BE-5F38-9A4B-895D-31A53476CF4D}" type="CELLRANGE">
+                    <a:fld id="{4D281085-63E9-6346-86AC-25E297DBF99A}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -802,7 +926,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{9C50B368-677F-0342-A924-9328B0932E87}" type="CELLRANGE">
+                    <a:fld id="{7D48E022-42F5-CD43-9F1A-8432D17F6044}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -840,7 +964,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{A9F16355-48FE-5347-BB62-2DDC61B556F8}" type="CELLRANGE">
+                    <a:fld id="{45F3000F-062C-CA46-BBDC-DB203FA4CA90}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -926,7 +1050,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{15D1427E-FBD7-5344-A96C-7FCE48C2C21D}" type="CELLRANGE">
+                    <a:fld id="{CE9D4C57-00B3-B844-BC70-1154ACEDF37A}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1283,7 +1407,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{85900E62-36C8-D44B-853A-1F3BCEDD6771}" type="CELLRANGE">
+                    <a:fld id="{0A38EB78-3077-0A4A-8298-23721E8BDAD2}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1430,7 +1554,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{C9DB9298-BF26-8146-82A6-EE202BDF84EA}" type="CELLRANGE">
+                    <a:fld id="{DB21B7A5-2339-D943-9C26-4FAF7AC500FE}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1468,7 +1592,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{30F2430F-C393-9E4C-9CFE-C15C6AC06B6D}" type="CELLRANGE">
+                    <a:fld id="{7475E913-C979-DB47-859B-B9DC939F9EFD}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1695,7 +1819,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{1945CC53-7840-C94E-A225-5A193CB81F0C}" type="CELLRANGE">
+                    <a:fld id="{32460BE8-6491-C045-9AE9-1D1AAFA1FFFE}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1760,7 +1884,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{7A7BBFB0-14E8-E34A-9938-AFB48E712359}" type="CELLRANGE">
+                    <a:fld id="{F043B2E2-CCA6-A14E-B5C0-DB6D019CF3BD}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1825,7 +1949,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{EF3B390C-CACA-334C-8452-7107118C2863}" type="CELLRANGE">
+                    <a:fld id="{8FFE7925-18A2-F34A-83D4-F265CD64220C}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1998,7 +2122,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{F98FE3AC-ACFD-F647-A8DD-E3709DC4FA9A}" type="CELLRANGE">
+                    <a:fld id="{D22AE2E8-4C5B-1544-B050-47F1CF560318}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2036,7 +2160,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{FEB9EF0E-13C8-1C44-9C12-AB4636B51A80}" type="CELLRANGE">
+                    <a:fld id="{DCAE78ED-FB0E-8549-9035-5B7EBD865D9E}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2074,7 +2198,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{8C293FF3-7361-C142-875C-74E8A7628B0E}" type="CELLRANGE">
+                    <a:fld id="{3FF97032-7F8C-F044-B6BD-FFBDA0FD6020}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2112,7 +2236,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{0287557D-7E9D-7B45-9206-1A5E1457A82A}" type="CELLRANGE">
+                    <a:fld id="{F60498B6-12F0-1E4A-9C0C-CAC88D818BDF}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2171,7 +2295,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{F69E69A2-2E76-CC4A-871D-098FD4951080}" type="CELLRANGE">
+                    <a:fld id="{970C6B6B-05EC-594D-8865-0043AAD038EC}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2204,7 +2328,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{FAB8CCC1-19BD-A34F-BBD9-8EB973259D73}" type="CELLRANGE">
+                    <a:fld id="{B8031B3F-2A8D-854B-A65C-9491237E4DAD}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2237,7 +2361,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{1E8E91D7-1F77-674A-8AB9-E5E84C2A628B}" type="CELLRANGE">
+                    <a:fld id="{8A5164B5-C9B3-7E45-9268-E0D08FCFC24F}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2276,7 +2400,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{1EF93158-6AE1-4D4F-A5AF-A59D67C7F96E}" type="CELLRANGE">
+                    <a:fld id="{3EE93E78-928C-D24F-9EA6-8797CB5930AF}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2314,7 +2438,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{08DEB95F-0A03-C24D-A7F1-1F3A06AADB78}" type="CELLRANGE">
+                    <a:fld id="{F81D291B-48AD-3040-9AFF-25266519FA93}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2352,7 +2476,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{30EEAC4A-7C21-0449-A7A6-14BB54188BBD}" type="CELLRANGE">
+                    <a:fld id="{A4C72768-979D-1942-AE51-F57CFEE13F65}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2390,7 +2514,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{5FBDCD96-7780-364B-ACE8-13FE5792BBF3}" type="CELLRANGE">
+                    <a:fld id="{B69997EA-C664-6B46-A2E9-79794B835774}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2428,7 +2552,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{80B7E842-366E-6A44-87BE-F3D81840E863}" type="CELLRANGE">
+                    <a:fld id="{CFBF5032-0C6C-2B48-8B77-7C7063BD80B7}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2460,7 +2584,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{18CAAA5D-CF07-2B40-932D-00E3823FD53A}" type="CELLRANGE">
+                    <a:fld id="{ED0E5A43-1C62-494C-959B-B85CBC626F09}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2499,7 +2623,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{B800F083-7CA6-A142-9E4E-CE5A4FF5A427}" type="CELLRANGE">
+                    <a:fld id="{E579C7E3-9878-A747-9149-655B778E9312}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2537,7 +2661,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{6FE5BED5-E952-9F47-837B-78B6CF89E425}" type="CELLRANGE">
+                    <a:fld id="{FBD91E69-B4B6-0145-B5D6-ED8D80D63E74}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2575,7 +2699,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{5AA4F5C6-6898-3944-955D-3E8884E897E2}" type="CELLRANGE">
+                    <a:fld id="{B91284D2-181F-254D-8EF6-3808BF2C4571}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2607,7 +2731,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{4D6F9C73-8001-D14A-A056-5B98C177BFA5}" type="CELLRANGE">
+                    <a:fld id="{2699E9B9-BFE3-244F-8DCB-12A2BC564BFA}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2646,7 +2770,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{0CA0EF7B-13B4-3443-854C-7EC9A9C65235}" type="CELLRANGE">
+                    <a:fld id="{8B45687E-E685-F044-A649-B53A9F72BEC1}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2684,7 +2808,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{CAFC1FC2-B7FC-4E43-A02D-7BCCEF20B005}" type="CELLRANGE">
+                    <a:fld id="{D616DDEE-A09C-0D43-B1B7-408214A8D310}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2722,7 +2846,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{B35B0603-3F02-8449-8348-0D960B6D42CE}" type="CELLRANGE">
+                    <a:fld id="{B80E9ACA-1D7D-0440-8CFE-E9B5025AEC9B}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2760,7 +2884,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{9A2E7B67-874B-6042-A7E5-3689B199E793}" type="CELLRANGE">
+                    <a:fld id="{96983823-0C35-8643-865E-5543CCFD9248}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -3775,7 +3899,7 @@
             </a:r>
             <a:r>
               <a:rPr lang="en-US" baseline="0"/>
-              <a:t> Graph</a:t>
+              <a:t> Graph (E2:E10)</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -3849,7 +3973,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{FC975DD8-73AD-274B-8A59-DA59A33B28F2}" type="CELLRANGE">
+                    <a:fld id="{014DD38E-35F3-1C4C-92AA-4A2D6017F424}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -3882,7 +4006,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{5D82D4D9-7135-2F45-A13F-65AD2B2C537D}" type="CELLRANGE">
+                    <a:fld id="{B270C088-8471-D74D-B8E1-32A3D15C9881}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -3915,7 +4039,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{B97D85D5-6707-C840-B35E-5500F95248E2}" type="CELLRANGE">
+                    <a:fld id="{66F2485F-EE33-5845-AC12-DD37697D4931}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -3954,7 +4078,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{C5665415-58EE-B84F-A3B4-7F2646E1E741}" type="CELLRANGE">
+                    <a:fld id="{E7E0E91A-D151-7443-8AC9-565FD2BCC9F6}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -3986,7 +4110,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{4D158764-D98D-FD4C-B89F-564F3433425B}" type="CELLRANGE">
+                    <a:fld id="{BC690AF9-3F0F-BD4F-9DE5-4412F5FB9E6C}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -4025,7 +4149,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{09E5FCBC-A5BC-D342-BA33-C3881214EEF2}" type="CELLRANGE">
+                    <a:fld id="{4CB43EF8-72FB-FB4D-AE13-4D262CD1EE3C}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -4063,7 +4187,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{91905E96-31CE-B442-B120-751770AA62A9}" type="CELLRANGE">
+                    <a:fld id="{FE718F82-1BE3-6C42-B0C8-D071E8CF821B}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -4095,7 +4219,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{C4A46D10-6039-DF4E-9550-B319FC0987E0}" type="CELLRANGE">
+                    <a:fld id="{B019FAA5-3FAF-CA4F-B906-C1BDF88C5A38}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -4134,7 +4258,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{89012BB3-8AF8-A143-8AF9-9FF40C1FC64A}" type="CELLRANGE">
+                    <a:fld id="{84D0483D-98C7-2E4E-A55E-BAD45999A606}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -4270,7 +4394,7 @@
           </c:trendline>
           <c:xVal>
             <c:numRef>
-              <c:f>Subset!$B$2:$B$10</c:f>
+              <c:f>Subset!$F$2:$F$10</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="9"/>
@@ -4306,7 +4430,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Subset!$C$2:$C$10</c:f>
+              <c:f>Subset!$G$2:$G$10</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="9"/>
@@ -4344,7 +4468,7 @@
           <c:extLst>
             <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
               <c15:datalabelsRange>
-                <c15:f>Subset!$A$2:$A$10</c15:f>
+                <c15:f>Subset!$E$2:$E$10</c15:f>
                 <c15:dlblRangeCache>
                   <c:ptCount val="9"/>
                   <c:pt idx="0">
@@ -5814,16 +5938,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>360606</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>65262</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>43106</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>1762</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>807424</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>157221</xdr:rowOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>489924</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>93721</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -6174,7 +6298,7 @@
     <col min="1" max="1" width="8.83203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.1640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
@@ -6199,6 +6323,9 @@
       <c r="C2">
         <v>2.6552462526766498</v>
       </c>
+      <c r="D2" s="5" t="s">
+        <v>76</v>
+      </c>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
     </row>
@@ -6210,6 +6337,9 @@
       <c r="C3">
         <v>2.6495726495726402</v>
       </c>
+      <c r="D3" s="5" t="s">
+        <v>76</v>
+      </c>
       <c r="E3" s="1"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
@@ -6220,7 +6350,9 @@
       <c r="C4">
         <v>2.53061224489795</v>
       </c>
-      <c r="D4" s="1"/>
+      <c r="D4" s="5" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
@@ -6230,7 +6362,9 @@
       <c r="C5">
         <v>2.52032520325203</v>
       </c>
-      <c r="D5" s="1"/>
+      <c r="D5" s="5" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
@@ -6240,7 +6374,9 @@
       <c r="C6">
         <v>2.4750499001996</v>
       </c>
-      <c r="D6" s="1"/>
+      <c r="D6" s="5" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
@@ -6250,7 +6386,9 @@
       <c r="C7">
         <v>2.46520874751491</v>
       </c>
-      <c r="D7" s="1"/>
+      <c r="D7" s="5" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
@@ -6260,7 +6398,9 @@
       <c r="C8">
         <v>2.0910623946037101</v>
       </c>
-      <c r="D8" s="1"/>
+      <c r="D8" s="5" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
@@ -6270,7 +6410,9 @@
       <c r="C9">
         <v>2.0840336134453699</v>
       </c>
-      <c r="D9" s="1"/>
+      <c r="D9" s="5" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
@@ -6282,7 +6424,9 @@
       <c r="C10">
         <v>2.7740492170022302</v>
       </c>
-      <c r="D10" s="1"/>
+      <c r="D10" s="5" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
@@ -6294,7 +6438,9 @@
       <c r="C11">
         <v>2.79279279279279</v>
       </c>
-      <c r="D11" s="1"/>
+      <c r="D11" s="5" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
@@ -6306,7 +6452,9 @@
       <c r="C12">
         <v>2.7740492170022302</v>
       </c>
-      <c r="D12" s="1"/>
+      <c r="D12" s="5" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
@@ -6318,7 +6466,9 @@
       <c r="C13">
         <v>2.7678571428571401</v>
       </c>
-      <c r="D13" s="1"/>
+      <c r="D13" s="5" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
@@ -6328,7 +6478,9 @@
       <c r="C14">
         <v>2.7678571428571401</v>
       </c>
-      <c r="D14" s="1"/>
+      <c r="D14" s="5" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
@@ -6337,7 +6489,9 @@
       <c r="C15">
         <v>2.4505928853754901</v>
       </c>
-      <c r="D15" s="1"/>
+      <c r="D15" s="5" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
@@ -6349,7 +6503,9 @@
       <c r="C16">
         <v>2.6839826839826801</v>
       </c>
-      <c r="D16" s="1"/>
+      <c r="D16" s="5" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
@@ -6358,6 +6514,9 @@
       <c r="C17">
         <v>2.6666666666666599</v>
       </c>
+      <c r="D17" s="5" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
@@ -6366,6 +6525,9 @@
       <c r="C18">
         <v>2.4077669902912602</v>
       </c>
+      <c r="D18" s="5" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
@@ -6374,6 +6536,9 @@
       <c r="C19">
         <v>2.6215644820295898</v>
       </c>
+      <c r="D19" s="5" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
@@ -6382,6 +6547,9 @@
       <c r="C20">
         <v>2.59958071278826</v>
       </c>
+      <c r="D20" s="5" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
@@ -6390,6 +6558,9 @@
       <c r="C21">
         <v>2.6215644820295898</v>
       </c>
+      <c r="D21" s="5" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
@@ -6398,6 +6569,9 @@
       <c r="C22">
         <v>2.6839826839826801</v>
       </c>
+      <c r="D22" s="5" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
@@ -6406,6 +6580,9 @@
       <c r="C23">
         <v>2.67241379310344</v>
       </c>
+      <c r="D23" s="5" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
@@ -6414,6 +6591,9 @@
       <c r="C24">
         <v>2.6666666666666599</v>
       </c>
+      <c r="D24" s="5" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
@@ -6422,6 +6602,9 @@
       <c r="C25">
         <v>2.8054298642533899</v>
       </c>
+      <c r="D25" s="5" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
@@ -6430,6 +6613,9 @@
       <c r="C26">
         <v>2.3352165725047</v>
       </c>
+      <c r="D26" s="5" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
@@ -6438,6 +6624,9 @@
       <c r="C27">
         <v>2.2878228782287802</v>
       </c>
+      <c r="D27" s="5" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
@@ -6446,6 +6635,9 @@
       <c r="C28">
         <v>2.5726141078838101</v>
       </c>
+      <c r="D28" s="5" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
@@ -6457,7 +6649,9 @@
       <c r="C29">
         <v>3.1392405063291098</v>
       </c>
-      <c r="D29" s="1"/>
+      <c r="D29" s="5" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
@@ -6466,6 +6660,9 @@
       <c r="C30">
         <v>3.1234256926952102</v>
       </c>
+      <c r="D30" s="5" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
@@ -6474,6 +6671,9 @@
       <c r="C31">
         <v>3.08457711442786</v>
       </c>
+      <c r="D31" s="5" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
@@ -6482,6 +6682,9 @@
       <c r="C32">
         <v>2.5357873210633901</v>
       </c>
+      <c r="D32" s="5" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
@@ -6490,6 +6693,9 @@
       <c r="C33">
         <v>2.7678571428571401</v>
       </c>
+      <c r="D33" s="5" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
@@ -6501,7 +6707,9 @@
       <c r="C34">
         <v>2.7555555555555502</v>
       </c>
-      <c r="D34" s="1"/>
+      <c r="D34" s="5" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
@@ -6513,7 +6721,9 @@
       <c r="C35">
         <v>2.8571428571428501</v>
       </c>
-      <c r="D35" s="1"/>
+      <c r="D35" s="5" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
@@ -6522,6 +6732,9 @@
       <c r="C36">
         <v>3.2291666666666599</v>
       </c>
+      <c r="D36" s="5" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
@@ -6530,6 +6743,9 @@
       <c r="C37">
         <v>2.6781857451403801</v>
       </c>
+      <c r="D37" s="5" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
@@ -6538,6 +6754,9 @@
       <c r="C38">
         <v>2.6271186440677901</v>
       </c>
+      <c r="D38" s="5" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
@@ -6546,6 +6765,9 @@
       <c r="C39">
         <v>2.31343283582089</v>
       </c>
+      <c r="D39" s="5" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
@@ -6554,6 +6776,9 @@
       <c r="C40">
         <v>2.1869488536155202</v>
       </c>
+      <c r="D40" s="5" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
@@ -6562,6 +6787,9 @@
       <c r="C41">
         <v>2.7678571428571401</v>
       </c>
+      <c r="D41" s="5" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
@@ -6570,6 +6798,9 @@
       <c r="C42">
         <v>2.7740492170022302</v>
       </c>
+      <c r="D42" s="5" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
@@ -6581,7 +6812,9 @@
       <c r="C43">
         <v>2.7678571428571401</v>
       </c>
-      <c r="D43" s="1"/>
+      <c r="D43" s="5" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
@@ -6590,6 +6823,9 @@
       <c r="C44">
         <v>2.7678571428571401</v>
       </c>
+      <c r="D44" s="5" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
@@ -6601,7 +6837,9 @@
       <c r="C45">
         <v>2.7616926503340702</v>
       </c>
-      <c r="D45" s="1"/>
+      <c r="D45" s="5" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
@@ -6610,6 +6848,9 @@
       <c r="C46">
         <v>2.7678571428571401</v>
       </c>
+      <c r="D46" s="5" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
@@ -6621,7 +6862,9 @@
       <c r="C47">
         <v>2.7678571428571401</v>
       </c>
-      <c r="D47" s="1"/>
+      <c r="D47" s="5" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
@@ -6630,6 +6873,9 @@
       <c r="C48">
         <v>2.6050420168067201</v>
       </c>
+      <c r="D48" s="5" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="s">
@@ -6638,6 +6884,9 @@
       <c r="C49">
         <v>2.5726141078838101</v>
       </c>
+      <c r="D49" s="5" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="s">
@@ -6646,6 +6895,9 @@
       <c r="C50">
         <v>2.6271186440677901</v>
       </c>
+      <c r="D50" s="5" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
@@ -6654,6 +6906,9 @@
       <c r="C51">
         <v>2.6956521739130399</v>
       </c>
+      <c r="D51" s="5" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A52" s="1" t="s">
@@ -6662,6 +6917,9 @@
       <c r="C52">
         <v>2.4409448818897599</v>
       </c>
+      <c r="D52" s="5" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
@@ -6673,7 +6931,9 @@
       <c r="C53">
         <v>2.6105263157894698</v>
       </c>
-      <c r="D53" s="1"/>
+      <c r="D53" s="5" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
@@ -6685,7 +6945,9 @@
       <c r="C54">
         <v>2.5462012320328502</v>
       </c>
-      <c r="D54" s="1"/>
+      <c r="D54" s="5" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
@@ -6697,7 +6959,9 @@
       <c r="C55">
         <v>2.6552462526766498</v>
       </c>
-      <c r="D55" s="1"/>
+      <c r="D55" s="5" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
@@ -6709,7 +6973,9 @@
       <c r="C56">
         <v>2.82460136674259</v>
       </c>
-      <c r="D56" s="1"/>
+      <c r="D56" s="5" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A57" s="1" t="s">
@@ -6718,6 +6984,9 @@
       <c r="C57">
         <v>2.6781857451403801</v>
       </c>
+      <c r="D57" s="5" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
@@ -6729,7 +6998,9 @@
       <c r="C58">
         <v>2.2222222222222201</v>
       </c>
-      <c r="D58" s="1"/>
+      <c r="D58" s="5" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
@@ -6741,7 +7012,9 @@
       <c r="C59">
         <v>2.2752293577981599</v>
       </c>
-      <c r="D59" s="1"/>
+      <c r="D59" s="5" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
@@ -6753,7 +7026,9 @@
       <c r="C60">
         <v>2.1342512908777902</v>
       </c>
-      <c r="D60" s="1"/>
+      <c r="D60" s="5" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
@@ -6765,7 +7040,9 @@
       <c r="C61">
         <v>2.1830985915492902</v>
       </c>
-      <c r="D61" s="1"/>
+      <c r="D61" s="5" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
@@ -6777,7 +7054,9 @@
       <c r="C62">
         <v>2.13793103448275</v>
       </c>
-      <c r="D62" s="1"/>
+      <c r="D62" s="5" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
@@ -6789,7 +7068,9 @@
       <c r="C63">
         <v>2.6215644820295898</v>
       </c>
-      <c r="D63" s="1"/>
+      <c r="D63" s="5" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
@@ -6801,7 +7082,9 @@
       <c r="C64">
         <v>2.7312775330396399</v>
       </c>
-      <c r="D64" s="1"/>
+      <c r="D64" s="5" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
@@ -6813,7 +7096,9 @@
       <c r="C65">
         <v>2.6105263157894698</v>
       </c>
-      <c r="D65" s="1"/>
+      <c r="D65" s="5" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
@@ -6825,7 +7110,9 @@
       <c r="C66">
         <v>2.04283360790774</v>
       </c>
-      <c r="D66" s="1"/>
+      <c r="D66" s="5" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
@@ -6837,7 +7124,9 @@
       <c r="C67">
         <v>2.0981387478849398</v>
       </c>
-      <c r="D67" s="1"/>
+      <c r="D67" s="5" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
@@ -6849,7 +7138,9 @@
       <c r="C68">
         <v>2.0361247947454801</v>
       </c>
-      <c r="D68" s="1"/>
+      <c r="D68" s="5" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
@@ -6861,7 +7152,9 @@
       <c r="C69">
         <v>2.39845261121856</v>
       </c>
-      <c r="D69" s="1"/>
+      <c r="D69" s="5" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
@@ -6873,7 +7166,9 @@
       <c r="C70">
         <v>2.3484848484848402</v>
       </c>
-      <c r="D70" s="1"/>
+      <c r="D70" s="5" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
@@ -6885,7 +7180,9 @@
       <c r="C71">
         <v>2.8770301624129901</v>
       </c>
-      <c r="D71" s="1"/>
+      <c r="D71" s="5" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
@@ -6897,7 +7194,9 @@
       <c r="C72">
         <v>2.8770301624129901</v>
       </c>
-      <c r="D72" s="1"/>
+      <c r="D72" s="5" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
@@ -6909,7 +7208,9 @@
       <c r="C73">
         <v>2.8117913832199499</v>
       </c>
-      <c r="D73" s="1"/>
+      <c r="D73" s="5" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
@@ -6921,7 +7222,9 @@
       <c r="C74">
         <v>2.82460136674259</v>
       </c>
-      <c r="D74" s="1"/>
+      <c r="D74" s="5" t="s">
+        <v>79</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -6932,120 +7235,929 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD3992E0-094E-8A42-B323-007503EE2A7D}">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:G74"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.5" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" t="s">
         <v>74</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>2.6552462526766498</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B2" s="3">
+      <c r="F2" s="3">
         <v>2.8054299999999999</v>
       </c>
-      <c r="C2" s="3">
+      <c r="G2" s="3">
         <v>0.179053136</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A3" s="2" t="s">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>2.6495726495726402</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B3" s="4">
+      <c r="F3" s="4">
         <v>2.2878229999999999</v>
       </c>
-      <c r="C3" s="4">
+      <c r="G3" s="4">
         <v>2.024669158</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" s="2" t="s">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>2.53061224489795</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B4" s="3">
+      <c r="F4" s="3">
         <v>2.3134329999999999</v>
       </c>
-      <c r="C4" s="3">
+      <c r="G4" s="3">
         <v>0.98336665700000003</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5" s="2" t="s">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>2.52032520325203</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="E5" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B5" s="3">
+      <c r="F5" s="3">
         <v>2.6050420000000001</v>
       </c>
-      <c r="C5" s="3">
+      <c r="G5" s="3">
         <v>0.51631367399999994</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A6" s="2" t="s">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>2.4750499001996</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="E6" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B6" s="4">
+      <c r="F6" s="4">
         <v>2.5726140000000002</v>
       </c>
-      <c r="C6" s="4">
+      <c r="G6" s="4">
         <v>2.2009162440000001</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A7" s="2" t="s">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>2.46520874751491</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="E7" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B7" s="3">
+      <c r="F7" s="3">
         <v>2.627119</v>
       </c>
-      <c r="C7" s="3">
+      <c r="G7" s="3">
         <v>0.80487891099999997</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A8" s="2" t="s">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>2.0910623946037101</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="E8" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B8" s="3">
+      <c r="F8" s="3">
         <v>2.6956519999999999</v>
       </c>
-      <c r="C8" s="3">
+      <c r="G8" s="3">
         <v>0.80487913499999997</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A9" s="2" t="s">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>2.0840336134453699</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="E9" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B9" s="4">
+      <c r="F9" s="4">
         <v>2.4409450000000001</v>
       </c>
-      <c r="C9" s="4">
+      <c r="G9" s="4">
         <v>2.14302729</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A10" s="2" t="s">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10">
+        <v>2.7740492170022302</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="E10" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B10" s="3">
+      <c r="F10" s="3">
         <v>2.655246</v>
       </c>
-      <c r="C10" s="3">
+      <c r="G10" s="3">
         <v>9.0716412999999996E-2</v>
       </c>
     </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11">
+        <v>2.79279279279279</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12">
+        <v>2.7740492170022302</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13">
+        <v>2.7678571428571401</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14">
+        <v>2.7678571428571401</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15">
+        <v>2.4505928853754901</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16">
+        <v>2.6839826839826801</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>16</v>
+      </c>
+      <c r="B17">
+        <v>2.6666666666666599</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>17</v>
+      </c>
+      <c r="B18">
+        <v>2.4077669902912602</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19">
+        <v>2.6215644820295898</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>19</v>
+      </c>
+      <c r="B20">
+        <v>2.59958071278826</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21">
+        <v>2.6215644820295898</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>21</v>
+      </c>
+      <c r="B22">
+        <v>2.6839826839826801</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>22</v>
+      </c>
+      <c r="B23">
+        <v>2.67241379310344</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>23</v>
+      </c>
+      <c r="B24">
+        <v>2.6666666666666599</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>24</v>
+      </c>
+      <c r="B25">
+        <v>2.8054298642533899</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>25</v>
+      </c>
+      <c r="B26">
+        <v>2.3352165725047</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>26</v>
+      </c>
+      <c r="B27">
+        <v>2.2878228782287802</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>27</v>
+      </c>
+      <c r="B28">
+        <v>2.5726141078838101</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>47</v>
+      </c>
+      <c r="B29">
+        <v>3.1392405063291098</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>28</v>
+      </c>
+      <c r="B30">
+        <v>3.1234256926952102</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>29</v>
+      </c>
+      <c r="B31">
+        <v>3.08457711442786</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>30</v>
+      </c>
+      <c r="B32">
+        <v>2.5357873210633901</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>31</v>
+      </c>
+      <c r="B33">
+        <v>2.7678571428571401</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>48</v>
+      </c>
+      <c r="B34">
+        <v>2.7555555555555502</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>49</v>
+      </c>
+      <c r="B35">
+        <v>2.8571428571428501</v>
+      </c>
+      <c r="C35" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>32</v>
+      </c>
+      <c r="B36">
+        <v>3.2291666666666599</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>33</v>
+      </c>
+      <c r="B37">
+        <v>2.6781857451403801</v>
+      </c>
+      <c r="C37" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>34</v>
+      </c>
+      <c r="B38">
+        <v>2.6271186440677901</v>
+      </c>
+      <c r="C38" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>35</v>
+      </c>
+      <c r="B39">
+        <v>2.31343283582089</v>
+      </c>
+      <c r="C39" s="5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>36</v>
+      </c>
+      <c r="B40">
+        <v>2.1869488536155202</v>
+      </c>
+      <c r="C40" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>37</v>
+      </c>
+      <c r="B41">
+        <v>2.7678571428571401</v>
+      </c>
+      <c r="C41" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>38</v>
+      </c>
+      <c r="B42">
+        <v>2.7740492170022302</v>
+      </c>
+      <c r="C42" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>50</v>
+      </c>
+      <c r="B43">
+        <v>2.7678571428571401</v>
+      </c>
+      <c r="C43" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>39</v>
+      </c>
+      <c r="B44">
+        <v>2.7678571428571401</v>
+      </c>
+      <c r="C44" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>57</v>
+      </c>
+      <c r="B45">
+        <v>2.7616926503340702</v>
+      </c>
+      <c r="C45" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>40</v>
+      </c>
+      <c r="B46">
+        <v>2.7678571428571401</v>
+      </c>
+      <c r="C46" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>51</v>
+      </c>
+      <c r="B47">
+        <v>2.7678571428571401</v>
+      </c>
+      <c r="C47" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>41</v>
+      </c>
+      <c r="B48">
+        <v>2.6050420168067201</v>
+      </c>
+      <c r="C48" s="5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>42</v>
+      </c>
+      <c r="B49">
+        <v>2.5726141078838101</v>
+      </c>
+      <c r="C49" s="5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>43</v>
+      </c>
+      <c r="B50">
+        <v>2.6271186440677901</v>
+      </c>
+      <c r="C50" s="5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>44</v>
+      </c>
+      <c r="B51">
+        <v>2.6956521739130399</v>
+      </c>
+      <c r="C51" s="5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>45</v>
+      </c>
+      <c r="B52">
+        <v>2.4409448818897599</v>
+      </c>
+      <c r="C52" s="5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
+        <v>58</v>
+      </c>
+      <c r="B53">
+        <v>2.6105263157894698</v>
+      </c>
+      <c r="C53" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
+        <v>59</v>
+      </c>
+      <c r="B54">
+        <v>2.5462012320328502</v>
+      </c>
+      <c r="C54" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
+        <v>60</v>
+      </c>
+      <c r="B55">
+        <v>2.6552462526766498</v>
+      </c>
+      <c r="C55" s="5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
+        <v>61</v>
+      </c>
+      <c r="B56">
+        <v>2.82460136674259</v>
+      </c>
+      <c r="C56" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
+        <v>46</v>
+      </c>
+      <c r="B57">
+        <v>2.6781857451403801</v>
+      </c>
+      <c r="C57" s="5" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
+        <v>52</v>
+      </c>
+      <c r="B58">
+        <v>2.2222222222222201</v>
+      </c>
+      <c r="C58" s="5" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
+        <v>53</v>
+      </c>
+      <c r="B59">
+        <v>2.2752293577981599</v>
+      </c>
+      <c r="C59" s="5" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A60" t="s">
+        <v>54</v>
+      </c>
+      <c r="B60">
+        <v>2.1342512908777902</v>
+      </c>
+      <c r="C60" s="5" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A61" t="s">
+        <v>55</v>
+      </c>
+      <c r="B61">
+        <v>2.1830985915492902</v>
+      </c>
+      <c r="C61" s="5" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A62" t="s">
+        <v>56</v>
+      </c>
+      <c r="B62">
+        <v>2.13793103448275</v>
+      </c>
+      <c r="C62" s="5" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A63" t="s">
+        <v>62</v>
+      </c>
+      <c r="B63">
+        <v>2.6215644820295898</v>
+      </c>
+      <c r="C63" s="5" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A64" t="s">
+        <v>46</v>
+      </c>
+      <c r="B64">
+        <v>2.7312775330396399</v>
+      </c>
+      <c r="C64" s="5" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A65" t="s">
+        <v>63</v>
+      </c>
+      <c r="B65">
+        <v>2.6105263157894698</v>
+      </c>
+      <c r="C65" s="5" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A66" t="s">
+        <v>64</v>
+      </c>
+      <c r="B66">
+        <v>2.04283360790774</v>
+      </c>
+      <c r="C66" s="5" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A67" t="s">
+        <v>65</v>
+      </c>
+      <c r="B67">
+        <v>2.0981387478849398</v>
+      </c>
+      <c r="C67" s="5" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A68" t="s">
+        <v>66</v>
+      </c>
+      <c r="B68">
+        <v>2.0361247947454801</v>
+      </c>
+      <c r="C68" s="5" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A69" t="s">
+        <v>67</v>
+      </c>
+      <c r="B69">
+        <v>2.39845261121856</v>
+      </c>
+      <c r="C69" s="5" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A70" t="s">
+        <v>68</v>
+      </c>
+      <c r="B70">
+        <v>2.3484848484848402</v>
+      </c>
+      <c r="C70" s="5" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A71" t="s">
+        <v>69</v>
+      </c>
+      <c r="B71">
+        <v>2.8770301624129901</v>
+      </c>
+      <c r="C71" s="5" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A72" t="s">
+        <v>70</v>
+      </c>
+      <c r="B72">
+        <v>2.8770301624129901</v>
+      </c>
+      <c r="C72" s="5" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A73" t="s">
+        <v>71</v>
+      </c>
+      <c r="B73">
+        <v>2.8117913832199499</v>
+      </c>
+      <c r="C73" s="5" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A74" t="s">
+        <v>72</v>
+      </c>
+      <c r="B74">
+        <v>2.82460136674259</v>
+      </c>
+      <c r="C74" s="5" t="s">
+        <v>79</v>
+      </c>
+    </row>
   </sheetData>
+  <conditionalFormatting sqref="C1:C1048576">
+    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="No Error Message">
+      <formula>NOT(ISERROR(SEARCH("No Error Message",C1)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Could not embed molecule">
+      <formula>NOT(ISERROR(SEARCH("Could not embed molecule",C1)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="0" priority="3" operator="containsText" text="Doesn't match templates">
+      <formula>NOT(ISERROR(SEARCH("Doesn't match templates",C1)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Rerun of singlet_triplet_gap script on corrected SMILES
</commit_message>
<xml_diff>
--- a/predicted_ee.xlsx
+++ b/predicted_ee.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zhuan08/Programming Projects/oled-project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71980309-8D09-8841-AEF8-B1DC5DD13656}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29243B97-566E-754E-8566-73799EBF3D77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="680" yWindow="740" windowWidth="28040" windowHeight="16840" xr2:uid="{2FDB0681-3AEB-6747-B8EB-32CB84415B37}"/>
+    <workbookView minimized="1" xWindow="680" yWindow="740" windowWidth="28040" windowHeight="16840" activeTab="1" xr2:uid="{2FDB0681-3AEB-6747-B8EB-32CB84415B37}"/>
   </bookViews>
   <sheets>
     <sheet name="Fullset" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="79">
   <si>
     <t>mol_id</t>
   </si>
@@ -270,13 +270,7 @@
     <t>Doesn't match templates</t>
   </si>
   <si>
-    <t>Could not embed molecule.</t>
-  </si>
-  <si>
     <t>No Error Message</t>
-  </si>
-  <si>
-    <t>Doesn't match templates}</t>
   </si>
   <si>
     <t xml:space="preserve">Could not embed molecule  </t>
@@ -376,7 +370,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="10">
+  <dxfs count="3">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -404,76 +398,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -850,7 +774,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{229006D0-909B-9D4A-BF3D-6107BD7EE258}" type="CELLRANGE">
+                    <a:fld id="{3D96DD04-FABE-704F-8A05-3906A49E78A4}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -888,7 +812,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{22E69E1E-12F2-EA46-825E-DE78818BAC4C}" type="CELLRANGE">
+                    <a:fld id="{00315D34-5EE8-C942-9618-668FA9608668}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -926,7 +850,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{225A82A3-38C3-2F4C-9505-048CDD03D26D}" type="CELLRANGE">
+                    <a:fld id="{31C8A2E0-A313-2541-B482-EF251FA4B9D9}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -964,7 +888,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{FB87303B-02D9-CE4B-8F50-DEFB3F819125}" type="CELLRANGE">
+                    <a:fld id="{8CD10A07-771B-A94B-9457-70D2479E7295}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1050,7 +974,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{15EFBCC6-886F-C94B-BBF6-199ED66099A7}" type="CELLRANGE">
+                    <a:fld id="{5CA13B0C-E9E5-D247-8485-1574FD0D01FC}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1407,7 +1331,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{D56E75DC-9C4A-C548-B202-61393FAC4516}" type="CELLRANGE">
+                    <a:fld id="{5444C74A-787D-0A44-90C7-480655E14EEA}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1554,7 +1478,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{1609D190-16D8-9F48-8DC4-2BB4925F04E0}" type="CELLRANGE">
+                    <a:fld id="{FC95B078-724C-1043-9603-D9D4BEA732DA}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1592,7 +1516,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{C4C5F691-E82B-9042-A43D-3917EAFDF559}" type="CELLRANGE">
+                    <a:fld id="{1A078CAD-A459-6D49-89B1-3AE02FCDFC0C}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1819,7 +1743,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{2A09BD28-3D26-D94F-8143-B1CBD2AEC733}" type="CELLRANGE">
+                    <a:fld id="{52BF39E3-1B28-674D-9239-E980048A636C}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1884,7 +1808,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{E85789A1-AE67-0C4D-9181-3C2577A6423C}" type="CELLRANGE">
+                    <a:fld id="{5F78E304-2408-5047-98A5-366BE98B3890}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1949,7 +1873,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{EB75F2A6-AAD6-5048-B0C9-3692A78D05D9}" type="CELLRANGE">
+                    <a:fld id="{911462FA-6406-7644-B8FD-0A3DE6A4E2FD}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2122,7 +2046,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{1ED2EE04-0C41-694C-8886-2B7F9C3F438C}" type="CELLRANGE">
+                    <a:fld id="{AD534723-4CDA-4B4F-90FF-C606C7602BC5}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2160,7 +2084,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{5BD89BDE-3B54-EC44-A382-586CD7E25F14}" type="CELLRANGE">
+                    <a:fld id="{BBC040F7-51C7-2F4F-93C9-B1A08C32045D}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2198,7 +2122,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{E1D99CE9-A0D3-1342-9773-467E3631D48C}" type="CELLRANGE">
+                    <a:fld id="{5188CA8F-D59A-8748-83BC-26610070BBEF}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2236,7 +2160,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{C483DAD3-6D72-EC40-B3C9-1CEAEC494BAA}" type="CELLRANGE">
+                    <a:fld id="{06B3906C-DDE4-1D45-9DFA-74FC75F1B731}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2295,7 +2219,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{FF12F3AC-6BAB-4F4E-8149-9B6285E4A126}" type="CELLRANGE">
+                    <a:fld id="{33C48293-DA96-F649-9DD6-DAC04BE7DE43}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2328,7 +2252,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{2701E762-3F21-2D42-B8B8-79789AAFF156}" type="CELLRANGE">
+                    <a:fld id="{66D68BF8-5739-2D4B-82DA-C4163F0A80C1}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2361,7 +2285,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{FCD77E45-2711-7448-9AEF-E9113CFEC31A}" type="CELLRANGE">
+                    <a:fld id="{4376A3F5-5B35-0648-BB9A-B09A0F0C929A}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2400,7 +2324,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{B8CABC6E-C9A1-B245-AB61-F88D1178EA0E}" type="CELLRANGE">
+                    <a:fld id="{1CAF75CE-2DCB-F443-AF6C-10AC5CED6C33}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2438,7 +2362,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{9A65CF4F-3B76-AE4F-9484-21C0B9BB9362}" type="CELLRANGE">
+                    <a:fld id="{23588EB5-3495-B84D-9F4C-16E6A22FD46F}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2476,7 +2400,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{41716539-3F18-BC46-B3D6-C4FB7EB35369}" type="CELLRANGE">
+                    <a:fld id="{332FA41C-FDF2-5044-B1B4-06AA36C63ED6}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2514,7 +2438,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{2F813E83-3E25-3546-85C7-42A0EFCF1BE6}" type="CELLRANGE">
+                    <a:fld id="{EC447570-A16C-FF4E-B7A3-3C0E7EC70F1F}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2552,7 +2476,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{B7BD11F3-80F2-0A42-A927-F54BFF72F6AF}" type="CELLRANGE">
+                    <a:fld id="{37C99A63-961F-524A-A621-3EDDD3A76A76}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2584,7 +2508,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{BE7D0CB3-1D35-BD4C-8F57-1A14108B89D0}" type="CELLRANGE">
+                    <a:fld id="{3F504945-A22F-6545-A421-C39E359C446B}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2623,7 +2547,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{AED3759E-510E-964B-97DC-AE572B480287}" type="CELLRANGE">
+                    <a:fld id="{7FD9DBBE-B636-1040-9F1C-D5D4229183DA}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2661,7 +2585,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{6936E857-E395-814A-B300-EA3C6D9D0162}" type="CELLRANGE">
+                    <a:fld id="{FDAEF48C-16A6-224F-9C78-E260B54D5521}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2699,7 +2623,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{38418643-1966-D642-8D87-D3240B26BF9E}" type="CELLRANGE">
+                    <a:fld id="{2D7345FB-0625-0B44-AA71-E7D924073DBE}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2731,7 +2655,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{97760775-A70F-6441-91C2-8A171C679CF2}" type="CELLRANGE">
+                    <a:fld id="{B98985A4-A40D-DE43-BB18-FF20956F6FBB}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2770,7 +2694,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{54242145-1ECF-FC46-A470-5A8425DA33B0}" type="CELLRANGE">
+                    <a:fld id="{3DDD78F3-32FE-1E45-B76E-C199223AF69F}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2808,7 +2732,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{0C9EE993-D8AA-4641-9DAE-50A4EFC2610D}" type="CELLRANGE">
+                    <a:fld id="{9638A435-7666-7746-82E4-93AE0A421EBA}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2846,7 +2770,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{E628C1A0-46C1-C14B-8C1A-5F6405CED98C}" type="CELLRANGE">
+                    <a:fld id="{23F36D41-2330-4449-BE90-ADC4EEBA255B}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2884,7 +2808,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{E176DE4D-4CB9-804F-AE8A-C204A8832690}" type="CELLRANGE">
+                    <a:fld id="{9D9487B7-EE6C-4244-8BBC-7D97BDDF9BD4}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -3973,7 +3897,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{B901ABEF-757F-7A4D-8140-44F5079A2748}" type="CELLRANGE">
+                    <a:fld id="{284BAC59-2FDD-364D-BB94-550EB118FB69}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -4006,7 +3930,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{995B6CFF-22AA-8345-BEE1-4E89EBA40D2C}" type="CELLRANGE">
+                    <a:fld id="{77E53A22-8ED4-9943-B5E7-5E769A3ECEAA}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -4039,7 +3963,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{D9C5890A-3D96-C549-9FD7-7D36A8580194}" type="CELLRANGE">
+                    <a:fld id="{6308855A-643F-024F-A889-2B2F62EEFFA4}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -4078,7 +4002,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{0EBBB58D-7424-2A41-978C-E8B5C4C95780}" type="CELLRANGE">
+                    <a:fld id="{64A9A9A6-E30E-EF41-A79C-66E56F11EB8C}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -4110,7 +4034,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{B33FD505-ACA7-8142-A315-B3E9E659323B}" type="CELLRANGE">
+                    <a:fld id="{A930E8EA-6B7B-7E41-B584-7216F27790FB}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -4149,7 +4073,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{AC85C595-98E4-6F47-B0BC-5A4437ED50E1}" type="CELLRANGE">
+                    <a:fld id="{0322DFCC-C05C-F344-B94B-D563457E248F}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -4187,7 +4111,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{F3694EC2-B545-D643-8BBB-1F90BCA1744E}" type="CELLRANGE">
+                    <a:fld id="{6D2EE69B-5834-E346-9D40-1AC9BBFA2768}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -4219,7 +4143,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{045B8FFB-DD71-6440-91F2-91A2E84A8E60}" type="CELLRANGE">
+                    <a:fld id="{89C86D13-F0A9-D34C-863F-61439A271E98}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -4258,7 +4182,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{A415F8F5-C718-B44E-9FE5-ECE2608C59A6}" type="CELLRANGE">
+                    <a:fld id="{E04086B1-61C8-8C43-8351-034BB023C366}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -5897,16 +5821,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>55667</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>194060</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1185967</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>130560</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>560699</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>134715</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>725799</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>71215</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -5939,15 +5863,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>43106</xdr:colOff>
+      <xdr:colOff>5006</xdr:colOff>
       <xdr:row>11</xdr:row>
-      <xdr:rowOff>1762</xdr:rowOff>
+      <xdr:rowOff>14462</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>489924</xdr:colOff>
+      <xdr:colOff>451824</xdr:colOff>
       <xdr:row>24</xdr:row>
-      <xdr:rowOff>93721</xdr:rowOff>
+      <xdr:rowOff>106421</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -6298,7 +6222,7 @@
     <col min="1" max="1" width="8.83203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.1640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
@@ -6311,9 +6235,6 @@
       <c r="C1" t="s">
         <v>74</v>
       </c>
-      <c r="D1" t="s">
-        <v>75</v>
-      </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
@@ -6323,9 +6244,7 @@
       <c r="C2">
         <v>2.6552462526766498</v>
       </c>
-      <c r="D2" s="5" t="s">
-        <v>76</v>
-      </c>
+      <c r="D2" s="5"/>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
     </row>
@@ -6337,9 +6256,7 @@
       <c r="C3">
         <v>2.6495726495726402</v>
       </c>
-      <c r="D3" s="5" t="s">
-        <v>76</v>
-      </c>
+      <c r="D3" s="5"/>
       <c r="E3" s="1"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
@@ -6350,9 +6267,7 @@
       <c r="C4">
         <v>2.53061224489795</v>
       </c>
-      <c r="D4" s="5" t="s">
-        <v>76</v>
-      </c>
+      <c r="D4" s="5"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
@@ -6362,9 +6277,7 @@
       <c r="C5">
         <v>2.52032520325203</v>
       </c>
-      <c r="D5" s="5" t="s">
-        <v>76</v>
-      </c>
+      <c r="D5" s="5"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
@@ -6374,9 +6287,7 @@
       <c r="C6">
         <v>2.4750499001996</v>
       </c>
-      <c r="D6" s="5" t="s">
-        <v>76</v>
-      </c>
+      <c r="D6" s="5"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
@@ -6386,9 +6297,7 @@
       <c r="C7">
         <v>2.46520874751491</v>
       </c>
-      <c r="D7" s="5" t="s">
-        <v>76</v>
-      </c>
+      <c r="D7" s="5"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
@@ -6398,9 +6307,7 @@
       <c r="C8">
         <v>2.0910623946037101</v>
       </c>
-      <c r="D8" s="5" t="s">
-        <v>76</v>
-      </c>
+      <c r="D8" s="5"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
@@ -6410,9 +6317,7 @@
       <c r="C9">
         <v>2.0840336134453699</v>
       </c>
-      <c r="D9" s="5" t="s">
-        <v>76</v>
-      </c>
+      <c r="D9" s="5"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
@@ -6424,9 +6329,7 @@
       <c r="C10">
         <v>2.7740492170022302</v>
       </c>
-      <c r="D10" s="5" t="s">
-        <v>77</v>
-      </c>
+      <c r="D10" s="5"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
@@ -6438,9 +6341,7 @@
       <c r="C11">
         <v>2.79279279279279</v>
       </c>
-      <c r="D11" s="5" t="s">
-        <v>77</v>
-      </c>
+      <c r="D11" s="5"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
@@ -6452,9 +6353,7 @@
       <c r="C12">
         <v>2.7740492170022302</v>
       </c>
-      <c r="D12" s="5" t="s">
-        <v>77</v>
-      </c>
+      <c r="D12" s="5"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
@@ -6466,9 +6365,7 @@
       <c r="C13">
         <v>2.7678571428571401</v>
       </c>
-      <c r="D13" s="5" t="s">
-        <v>77</v>
-      </c>
+      <c r="D13" s="5"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
@@ -6478,9 +6375,7 @@
       <c r="C14">
         <v>2.7678571428571401</v>
       </c>
-      <c r="D14" s="5" t="s">
-        <v>77</v>
-      </c>
+      <c r="D14" s="5"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
@@ -6489,9 +6384,7 @@
       <c r="C15">
         <v>2.4505928853754901</v>
       </c>
-      <c r="D15" s="5" t="s">
-        <v>77</v>
-      </c>
+      <c r="D15" s="5"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
@@ -6503,9 +6396,7 @@
       <c r="C16">
         <v>2.6839826839826801</v>
       </c>
-      <c r="D16" s="5" t="s">
-        <v>77</v>
-      </c>
+      <c r="D16" s="5"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
@@ -6514,9 +6405,7 @@
       <c r="C17">
         <v>2.6666666666666599</v>
       </c>
-      <c r="D17" s="5" t="s">
-        <v>77</v>
-      </c>
+      <c r="D17" s="5"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
@@ -6525,9 +6414,7 @@
       <c r="C18">
         <v>2.4077669902912602</v>
       </c>
-      <c r="D18" s="5" t="s">
-        <v>77</v>
-      </c>
+      <c r="D18" s="5"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
@@ -6536,9 +6423,7 @@
       <c r="C19">
         <v>2.6215644820295898</v>
       </c>
-      <c r="D19" s="5" t="s">
-        <v>77</v>
-      </c>
+      <c r="D19" s="5"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
@@ -6547,9 +6432,7 @@
       <c r="C20">
         <v>2.59958071278826</v>
       </c>
-      <c r="D20" s="5" t="s">
-        <v>77</v>
-      </c>
+      <c r="D20" s="5"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
@@ -6558,9 +6441,7 @@
       <c r="C21">
         <v>2.6215644820295898</v>
       </c>
-      <c r="D21" s="5" t="s">
-        <v>77</v>
-      </c>
+      <c r="D21" s="5"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
@@ -6569,9 +6450,7 @@
       <c r="C22">
         <v>2.6839826839826801</v>
       </c>
-      <c r="D22" s="5" t="s">
-        <v>77</v>
-      </c>
+      <c r="D22" s="5"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
@@ -6580,9 +6459,7 @@
       <c r="C23">
         <v>2.67241379310344</v>
       </c>
-      <c r="D23" s="5" t="s">
-        <v>77</v>
-      </c>
+      <c r="D23" s="5"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
@@ -6591,9 +6468,7 @@
       <c r="C24">
         <v>2.6666666666666599</v>
       </c>
-      <c r="D24" s="5" t="s">
-        <v>77</v>
-      </c>
+      <c r="D24" s="5"/>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
@@ -6602,9 +6477,7 @@
       <c r="C25">
         <v>2.8054298642533899</v>
       </c>
-      <c r="D25" s="5" t="s">
-        <v>78</v>
-      </c>
+      <c r="D25" s="5"/>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
@@ -6613,9 +6486,7 @@
       <c r="C26">
         <v>2.3352165725047</v>
       </c>
-      <c r="D26" s="5" t="s">
-        <v>77</v>
-      </c>
+      <c r="D26" s="5"/>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
@@ -6624,9 +6495,7 @@
       <c r="C27">
         <v>2.2878228782287802</v>
       </c>
-      <c r="D27" s="5" t="s">
-        <v>78</v>
-      </c>
+      <c r="D27" s="5"/>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
@@ -6635,9 +6504,7 @@
       <c r="C28">
         <v>2.5726141078838101</v>
       </c>
-      <c r="D28" s="5" t="s">
-        <v>77</v>
-      </c>
+      <c r="D28" s="5"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
@@ -6649,9 +6516,7 @@
       <c r="C29">
         <v>3.1392405063291098</v>
       </c>
-      <c r="D29" s="5" t="s">
-        <v>77</v>
-      </c>
+      <c r="D29" s="5"/>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
@@ -6660,9 +6525,7 @@
       <c r="C30">
         <v>3.1234256926952102</v>
       </c>
-      <c r="D30" s="5" t="s">
-        <v>77</v>
-      </c>
+      <c r="D30" s="5"/>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
@@ -6671,9 +6534,7 @@
       <c r="C31">
         <v>3.08457711442786</v>
       </c>
-      <c r="D31" s="5" t="s">
-        <v>77</v>
-      </c>
+      <c r="D31" s="5"/>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
@@ -6682,9 +6543,7 @@
       <c r="C32">
         <v>2.5357873210633901</v>
       </c>
-      <c r="D32" s="5" t="s">
-        <v>77</v>
-      </c>
+      <c r="D32" s="5"/>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
@@ -6693,9 +6552,7 @@
       <c r="C33">
         <v>2.7678571428571401</v>
       </c>
-      <c r="D33" s="5" t="s">
-        <v>77</v>
-      </c>
+      <c r="D33" s="5"/>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
@@ -6707,9 +6564,7 @@
       <c r="C34">
         <v>2.7555555555555502</v>
       </c>
-      <c r="D34" s="5" t="s">
-        <v>77</v>
-      </c>
+      <c r="D34" s="5"/>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
@@ -6721,9 +6576,7 @@
       <c r="C35">
         <v>2.8571428571428501</v>
       </c>
-      <c r="D35" s="5" t="s">
-        <v>77</v>
-      </c>
+      <c r="D35" s="5"/>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
@@ -6732,9 +6585,7 @@
       <c r="C36">
         <v>3.2291666666666599</v>
       </c>
-      <c r="D36" s="5" t="s">
-        <v>77</v>
-      </c>
+      <c r="D36" s="5"/>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
@@ -6743,9 +6594,7 @@
       <c r="C37">
         <v>2.6781857451403801</v>
       </c>
-      <c r="D37" s="5" t="s">
-        <v>77</v>
-      </c>
+      <c r="D37" s="5"/>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
@@ -6754,9 +6603,7 @@
       <c r="C38">
         <v>2.6271186440677901</v>
       </c>
-      <c r="D38" s="5" t="s">
-        <v>77</v>
-      </c>
+      <c r="D38" s="5"/>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
@@ -6765,9 +6612,7 @@
       <c r="C39">
         <v>2.31343283582089</v>
       </c>
-      <c r="D39" s="5" t="s">
-        <v>78</v>
-      </c>
+      <c r="D39" s="5"/>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
@@ -6776,9 +6621,7 @@
       <c r="C40">
         <v>2.1869488536155202</v>
       </c>
-      <c r="D40" s="5" t="s">
-        <v>77</v>
-      </c>
+      <c r="D40" s="5"/>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
@@ -6787,9 +6630,7 @@
       <c r="C41">
         <v>2.7678571428571401</v>
       </c>
-      <c r="D41" s="5" t="s">
-        <v>77</v>
-      </c>
+      <c r="D41" s="5"/>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
@@ -6798,9 +6639,7 @@
       <c r="C42">
         <v>2.7740492170022302</v>
       </c>
-      <c r="D42" s="5" t="s">
-        <v>77</v>
-      </c>
+      <c r="D42" s="5"/>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
@@ -6812,9 +6651,7 @@
       <c r="C43">
         <v>2.7678571428571401</v>
       </c>
-      <c r="D43" s="5" t="s">
-        <v>77</v>
-      </c>
+      <c r="D43" s="5"/>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
@@ -6823,9 +6660,7 @@
       <c r="C44">
         <v>2.7678571428571401</v>
       </c>
-      <c r="D44" s="5" t="s">
-        <v>77</v>
-      </c>
+      <c r="D44" s="5"/>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
@@ -6837,9 +6672,7 @@
       <c r="C45">
         <v>2.7616926503340702</v>
       </c>
-      <c r="D45" s="5" t="s">
-        <v>77</v>
-      </c>
+      <c r="D45" s="5"/>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
@@ -6848,9 +6681,7 @@
       <c r="C46">
         <v>2.7678571428571401</v>
       </c>
-      <c r="D46" s="5" t="s">
-        <v>77</v>
-      </c>
+      <c r="D46" s="5"/>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
@@ -6862,9 +6693,7 @@
       <c r="C47">
         <v>2.7678571428571401</v>
       </c>
-      <c r="D47" s="5" t="s">
-        <v>77</v>
-      </c>
+      <c r="D47" s="5"/>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
@@ -6873,9 +6702,7 @@
       <c r="C48">
         <v>2.6050420168067201</v>
       </c>
-      <c r="D48" s="5" t="s">
-        <v>78</v>
-      </c>
+      <c r="D48" s="5"/>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="s">
@@ -6884,9 +6711,7 @@
       <c r="C49">
         <v>2.5726141078838101</v>
       </c>
-      <c r="D49" s="5" t="s">
-        <v>78</v>
-      </c>
+      <c r="D49" s="5"/>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="s">
@@ -6895,9 +6720,7 @@
       <c r="C50">
         <v>2.6271186440677901</v>
       </c>
-      <c r="D50" s="5" t="s">
-        <v>78</v>
-      </c>
+      <c r="D50" s="5"/>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
@@ -6906,9 +6729,7 @@
       <c r="C51">
         <v>2.6956521739130399</v>
       </c>
-      <c r="D51" s="5" t="s">
-        <v>78</v>
-      </c>
+      <c r="D51" s="5"/>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A52" s="1" t="s">
@@ -6917,9 +6738,7 @@
       <c r="C52">
         <v>2.4409448818897599</v>
       </c>
-      <c r="D52" s="5" t="s">
-        <v>78</v>
-      </c>
+      <c r="D52" s="5"/>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
@@ -6931,9 +6750,7 @@
       <c r="C53">
         <v>2.6105263157894698</v>
       </c>
-      <c r="D53" s="5" t="s">
-        <v>77</v>
-      </c>
+      <c r="D53" s="5"/>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
@@ -6945,9 +6762,7 @@
       <c r="C54">
         <v>2.5462012320328502</v>
       </c>
-      <c r="D54" s="5" t="s">
-        <v>77</v>
-      </c>
+      <c r="D54" s="5"/>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
@@ -6959,9 +6774,7 @@
       <c r="C55">
         <v>2.6552462526766498</v>
       </c>
-      <c r="D55" s="5" t="s">
-        <v>78</v>
-      </c>
+      <c r="D55" s="5"/>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
@@ -6973,9 +6786,7 @@
       <c r="C56">
         <v>2.82460136674259</v>
       </c>
-      <c r="D56" s="5" t="s">
-        <v>77</v>
-      </c>
+      <c r="D56" s="5"/>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A57" s="1" t="s">
@@ -6984,9 +6795,7 @@
       <c r="C57">
         <v>2.6781857451403801</v>
       </c>
-      <c r="D57" s="5" t="s">
-        <v>76</v>
-      </c>
+      <c r="D57" s="5"/>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
@@ -6998,9 +6807,7 @@
       <c r="C58">
         <v>2.2222222222222201</v>
       </c>
-      <c r="D58" s="5" t="s">
-        <v>76</v>
-      </c>
+      <c r="D58" s="5"/>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
@@ -7012,9 +6819,7 @@
       <c r="C59">
         <v>2.2752293577981599</v>
       </c>
-      <c r="D59" s="5" t="s">
-        <v>76</v>
-      </c>
+      <c r="D59" s="5"/>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
@@ -7026,9 +6831,7 @@
       <c r="C60">
         <v>2.1342512908777902</v>
       </c>
-      <c r="D60" s="5" t="s">
-        <v>76</v>
-      </c>
+      <c r="D60" s="5"/>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
@@ -7040,9 +6843,7 @@
       <c r="C61">
         <v>2.1830985915492902</v>
       </c>
-      <c r="D61" s="5" t="s">
-        <v>76</v>
-      </c>
+      <c r="D61" s="5"/>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
@@ -7054,9 +6855,7 @@
       <c r="C62">
         <v>2.13793103448275</v>
       </c>
-      <c r="D62" s="5" t="s">
-        <v>76</v>
-      </c>
+      <c r="D62" s="5"/>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
@@ -7068,9 +6867,7 @@
       <c r="C63">
         <v>2.6215644820295898</v>
       </c>
-      <c r="D63" s="5" t="s">
-        <v>76</v>
-      </c>
+      <c r="D63" s="5"/>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
@@ -7082,9 +6879,7 @@
       <c r="C64">
         <v>2.7312775330396399</v>
       </c>
-      <c r="D64" s="5" t="s">
-        <v>76</v>
-      </c>
+      <c r="D64" s="5"/>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
@@ -7096,9 +6891,7 @@
       <c r="C65">
         <v>2.6105263157894698</v>
       </c>
-      <c r="D65" s="5" t="s">
-        <v>76</v>
-      </c>
+      <c r="D65" s="5"/>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
@@ -7110,9 +6903,7 @@
       <c r="C66">
         <v>2.04283360790774</v>
       </c>
-      <c r="D66" s="5" t="s">
-        <v>76</v>
-      </c>
+      <c r="D66" s="5"/>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
@@ -7124,9 +6915,7 @@
       <c r="C67">
         <v>2.0981387478849398</v>
       </c>
-      <c r="D67" s="5" t="s">
-        <v>76</v>
-      </c>
+      <c r="D67" s="5"/>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
@@ -7138,9 +6927,7 @@
       <c r="C68">
         <v>2.0361247947454801</v>
       </c>
-      <c r="D68" s="5" t="s">
-        <v>76</v>
-      </c>
+      <c r="D68" s="5"/>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
@@ -7152,9 +6939,7 @@
       <c r="C69">
         <v>2.39845261121856</v>
       </c>
-      <c r="D69" s="5" t="s">
-        <v>76</v>
-      </c>
+      <c r="D69" s="5"/>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
@@ -7166,9 +6951,7 @@
       <c r="C70">
         <v>2.3484848484848402</v>
       </c>
-      <c r="D70" s="5" t="s">
-        <v>76</v>
-      </c>
+      <c r="D70" s="5"/>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
@@ -7180,9 +6963,7 @@
       <c r="C71">
         <v>2.8770301624129901</v>
       </c>
-      <c r="D71" s="5" t="s">
-        <v>76</v>
-      </c>
+      <c r="D71" s="5"/>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
@@ -7194,9 +6975,7 @@
       <c r="C72">
         <v>2.8770301624129901</v>
       </c>
-      <c r="D72" s="5" t="s">
-        <v>76</v>
-      </c>
+      <c r="D72" s="5"/>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
@@ -7208,9 +6987,7 @@
       <c r="C73">
         <v>2.8117913832199499</v>
       </c>
-      <c r="D73" s="5" t="s">
-        <v>76</v>
-      </c>
+      <c r="D73" s="5"/>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
@@ -7222,9 +6999,7 @@
       <c r="C74">
         <v>2.82460136674259</v>
       </c>
-      <c r="D74" s="5" t="s">
-        <v>79</v>
-      </c>
+      <c r="D74" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -7430,7 +7205,7 @@
         <v>2.7740492170022302</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>60</v>
@@ -7450,7 +7225,7 @@
         <v>2.79279279279279</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
@@ -7461,7 +7236,7 @@
         <v>2.7740492170022302</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
@@ -7472,7 +7247,7 @@
         <v>2.7678571428571401</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
@@ -7483,7 +7258,7 @@
         <v>2.7678571428571401</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
@@ -7494,7 +7269,7 @@
         <v>2.4505928853754901</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
@@ -7505,7 +7280,7 @@
         <v>2.6839826839826801</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
@@ -7516,7 +7291,7 @@
         <v>2.6666666666666599</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
@@ -7527,7 +7302,7 @@
         <v>2.4077669902912602</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
@@ -7538,7 +7313,7 @@
         <v>2.6215644820295898</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
@@ -7549,7 +7324,7 @@
         <v>2.59958071278826</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
@@ -7560,7 +7335,7 @@
         <v>2.6215644820295898</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
@@ -7571,7 +7346,7 @@
         <v>2.6839826839826801</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
@@ -7582,7 +7357,7 @@
         <v>2.67241379310344</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
@@ -7593,7 +7368,7 @@
         <v>2.6666666666666599</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
@@ -7604,7 +7379,7 @@
         <v>2.8054298642533899</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
@@ -7615,7 +7390,7 @@
         <v>2.3352165725047</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
@@ -7626,7 +7401,7 @@
         <v>2.2878228782287802</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.2">
@@ -7637,7 +7412,7 @@
         <v>2.5726141078838101</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.2">
@@ -7648,7 +7423,7 @@
         <v>3.1392405063291098</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.2">
@@ -7659,7 +7434,7 @@
         <v>3.1234256926952102</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.2">
@@ -7670,7 +7445,7 @@
         <v>3.08457711442786</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.2">
@@ -7681,7 +7456,7 @@
         <v>2.5357873210633901</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.2">
@@ -7692,7 +7467,7 @@
         <v>2.7678571428571401</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.2">
@@ -7703,7 +7478,7 @@
         <v>2.7555555555555502</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.2">
@@ -7714,7 +7489,7 @@
         <v>2.8571428571428501</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.2">
@@ -7725,7 +7500,7 @@
         <v>3.2291666666666599</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.2">
@@ -7736,7 +7511,7 @@
         <v>2.6781857451403801</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.2">
@@ -7747,7 +7522,7 @@
         <v>2.6271186440677901</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.2">
@@ -7758,7 +7533,7 @@
         <v>2.31343283582089</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.2">
@@ -7769,7 +7544,7 @@
         <v>2.1869488536155202</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.2">
@@ -7780,7 +7555,7 @@
         <v>2.7678571428571401</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.2">
@@ -7791,7 +7566,7 @@
         <v>2.7740492170022302</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.2">
@@ -7802,7 +7577,7 @@
         <v>2.7678571428571401</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.2">
@@ -7813,7 +7588,7 @@
         <v>2.7678571428571401</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.2">
@@ -7824,7 +7599,7 @@
         <v>2.7616926503340702</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.2">
@@ -7835,7 +7610,7 @@
         <v>2.7678571428571401</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.2">
@@ -7846,7 +7621,7 @@
         <v>2.7678571428571401</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.2">
@@ -7857,7 +7632,7 @@
         <v>2.6050420168067201</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.2">
@@ -7868,7 +7643,7 @@
         <v>2.5726141078838101</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.2">
@@ -7879,7 +7654,7 @@
         <v>2.6271186440677901</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.2">
@@ -7890,7 +7665,7 @@
         <v>2.6956521739130399</v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.2">
@@ -7901,7 +7676,7 @@
         <v>2.4409448818897599</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.2">
@@ -7912,7 +7687,7 @@
         <v>2.6105263157894698</v>
       </c>
       <c r="C53" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.2">
@@ -7923,7 +7698,7 @@
         <v>2.5462012320328502</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.2">
@@ -7934,7 +7709,7 @@
         <v>2.6552462526766498</v>
       </c>
       <c r="C55" s="5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.2">
@@ -7945,7 +7720,7 @@
         <v>2.82460136674259</v>
       </c>
       <c r="C56" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.2">
@@ -8143,7 +7918,7 @@
         <v>2.82460136674259</v>
       </c>
       <c r="C74" s="5" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Began to start separating singlet_triplet_gap script into two parts
</commit_message>
<xml_diff>
--- a/predicted_ee.xlsx
+++ b/predicted_ee.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zhuan08/Programming Projects/oled-project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FE99EAA-E66E-4B45-AC1A-72A566B9424E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47635C4A-8904-5942-8929-E88C47C8AA4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="680" yWindow="740" windowWidth="28040" windowHeight="16840" activeTab="1" xr2:uid="{2FDB0681-3AEB-6747-B8EB-32CB84415B37}"/>
+    <workbookView xWindow="680" yWindow="740" windowWidth="28040" windowHeight="16840" activeTab="2" xr2:uid="{2FDB0681-3AEB-6747-B8EB-32CB84415B37}"/>
   </bookViews>
   <sheets>
     <sheet name="Fullset" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="84">
   <si>
     <t>mol_id</t>
   </si>
@@ -296,6 +296,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0000"/>
+  </numFmts>
   <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -396,7 +399,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -406,7 +409,8 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -845,7 +849,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{B19A918B-2485-CE44-B4EC-5C990EE41F6C}" type="CELLRANGE">
+                    <a:fld id="{52298BA8-D77B-8C4E-BCE2-CBC9B5C91DB7}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -883,7 +887,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{733E518A-C90B-4A43-8889-20C1673C7593}" type="CELLRANGE">
+                    <a:fld id="{8D49DB9D-C64B-274B-915A-D9DF078DF63E}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -921,7 +925,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{F507560C-0E9C-154D-AFA9-46807A5A0B25}" type="CELLRANGE">
+                    <a:fld id="{67E58140-5A15-414C-BC8D-D6CE21687FD4}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -959,7 +963,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{A2F8FCCE-5ED0-2D40-9E88-4D41BF67DFFC}" type="CELLRANGE">
+                    <a:fld id="{027409EC-3BFA-2241-B681-8F46DA5FF988}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1045,7 +1049,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{89DB6B5A-400E-EB47-93E0-4342050D06B6}" type="CELLRANGE">
+                    <a:fld id="{BC06B8E0-B8DE-C24B-A519-D0B8BCF630EA}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1402,7 +1406,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{EFE8329C-F38B-504B-A861-F5B0FCAD4A4B}" type="CELLRANGE">
+                    <a:fld id="{BCA4E46A-05F6-E645-AA8A-0B1C0E282026}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1549,7 +1553,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{BE686C2D-003A-E24B-8B2D-D1478205E5E5}" type="CELLRANGE">
+                    <a:fld id="{0549D33B-A99A-1642-8FF1-DA3F6079AE74}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1587,7 +1591,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{38EEC392-0CF7-7C44-9A34-35FA3D20638B}" type="CELLRANGE">
+                    <a:fld id="{B9827EDE-1E5F-EF49-BA96-FF055F3755B9}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1814,7 +1818,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{BA055513-959B-FF4C-8C22-E3E8416BDE7E}" type="CELLRANGE">
+                    <a:fld id="{6D326EAC-B229-B548-AB24-EF58B1921AE2}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1879,7 +1883,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{9FCDAA32-CB7A-BD4D-BD41-1E1DD02B550D}" type="CELLRANGE">
+                    <a:fld id="{878BB8C5-86FF-6941-B4FD-E5F8E090A8CA}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1944,7 +1948,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{5CEC629B-2986-EE43-BDB9-2ED1C282BF89}" type="CELLRANGE">
+                    <a:fld id="{09F40E60-63D9-CC47-AC6B-8BAA7FAC77FE}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2117,7 +2121,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{107848A0-7073-5B4D-8996-7E4A806379C4}" type="CELLRANGE">
+                    <a:fld id="{80A32642-B9CD-B448-B7CF-B03C0E6D40D9}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2155,7 +2159,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{6D6DE508-02DE-2F40-951E-B06E6ACF849B}" type="CELLRANGE">
+                    <a:fld id="{F005BF63-8775-B54E-9021-97D48577A3CE}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2193,7 +2197,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{261FCD64-90FF-A04D-A2F7-32AFDAA5EE53}" type="CELLRANGE">
+                    <a:fld id="{FA6AD7CB-FC8E-E44B-AB81-DEA16E733ECC}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2231,7 +2235,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{3B062EDD-B81F-8D4B-8E51-4BF6FF383983}" type="CELLRANGE">
+                    <a:fld id="{F1476565-85C1-5A47-8440-4477CC33A5D6}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2290,7 +2294,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{C4740CAC-8E3B-1041-B8E4-E5725E690BC0}" type="CELLRANGE">
+                    <a:fld id="{8CA0AD66-FDA0-2949-9295-2174B48690FD}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2323,7 +2327,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{40EC6B52-BD8B-E941-98DB-355145ABEB0F}" type="CELLRANGE">
+                    <a:fld id="{004B0E47-2C6F-084C-B266-F530EE8CE60C}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2356,7 +2360,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{AD71621B-B8AB-EA45-8453-572677CD4B45}" type="CELLRANGE">
+                    <a:fld id="{7705A45A-CD1C-A24A-B272-46F4B6365DAD}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2395,7 +2399,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{ADD1866F-47F0-154E-9B05-B63E7DAB6AC0}" type="CELLRANGE">
+                    <a:fld id="{8CFE1E5A-B151-A244-8DBE-A42AC8B531C8}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2433,7 +2437,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{20587D1A-64E0-B34A-977B-AF78D9A30558}" type="CELLRANGE">
+                    <a:fld id="{5480B7BD-13AA-A440-B430-03A27C50B374}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2471,7 +2475,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{934675B9-FD7F-894B-A33D-78161DF1C32F}" type="CELLRANGE">
+                    <a:fld id="{23A1B921-452A-AF4A-8C59-BA0A28114909}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2509,7 +2513,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{1C53F5C4-FEF8-D14C-A56F-EE501FFD1CC6}" type="CELLRANGE">
+                    <a:fld id="{CF3E921F-9380-0F49-AEA9-DCB266218FD2}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2547,7 +2551,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{2F5602B7-D719-E445-957E-892C5A7DC3FD}" type="CELLRANGE">
+                    <a:fld id="{7FEF361B-EC5F-B64A-BB34-70192398F757}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2579,7 +2583,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{85208B5A-FC9D-9640-B220-DE97D84E6D09}" type="CELLRANGE">
+                    <a:fld id="{C15F531A-5975-644F-B9D8-207A2679DEE3}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2618,7 +2622,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{4DF4F1CF-2AA2-434C-8BBF-523A1B6B347B}" type="CELLRANGE">
+                    <a:fld id="{BA8DAB57-E6EC-ED4C-8E7F-C783D2D912DD}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2656,7 +2660,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{1957BD8E-1685-EC46-B1A9-FECE8CFC08F2}" type="CELLRANGE">
+                    <a:fld id="{CC73C4A7-E69B-2B47-920F-276E4A2F37A0}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2694,7 +2698,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{7D86CF8A-4F28-B141-8731-97D8C102B1D0}" type="CELLRANGE">
+                    <a:fld id="{A40AE722-6DBE-FF45-A861-5AFBEE2F923D}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2726,7 +2730,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{42393B9B-D45B-2A4C-A74B-E30CCDEE2794}" type="CELLRANGE">
+                    <a:fld id="{57993BF1-06ED-464E-B386-467463D57D51}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2765,7 +2769,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{E1EE2D91-EB53-5D49-9EDF-77326F561753}" type="CELLRANGE">
+                    <a:fld id="{F0131110-AEC9-5542-B12B-E500663085A3}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2803,7 +2807,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{92C9523A-18A8-F24F-8005-CB46F5FE97ED}" type="CELLRANGE">
+                    <a:fld id="{70B24EA4-387F-4D49-9F5B-14CB4BA7FC21}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2841,7 +2845,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{1D79FCA1-4E23-FD4F-A6D8-04A9339C629A}" type="CELLRANGE">
+                    <a:fld id="{671249F4-16FB-A541-AD5F-30006CC20A19}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2879,7 +2883,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{1876551C-1869-4543-9D9C-9F26E44C5C34}" type="CELLRANGE">
+                    <a:fld id="{482029A0-3370-B344-9513-D9C4A6CA2F1E}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -3968,7 +3972,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{AAED89AD-1061-C242-96DF-A5BC3FCCFCF4}" type="CELLRANGE">
+                    <a:fld id="{1AC90E69-0066-604B-87CE-EC2FB39AEAD9}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -4001,7 +4005,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{ABDF0F59-2578-5746-A5E2-18E4B369AA8E}" type="CELLRANGE">
+                    <a:fld id="{F165791C-BE19-C94A-9319-9C368FB3D56E}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -4034,7 +4038,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{FE47618A-8908-2043-A2B7-E9A304F97DE1}" type="CELLRANGE">
+                    <a:fld id="{40E0989A-ED09-E54B-8F97-D3AAB259DF1E}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -4073,7 +4077,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{01D3A284-6169-A54D-80C1-4023162832A8}" type="CELLRANGE">
+                    <a:fld id="{4B5AFDBE-A040-E149-B829-DB370FD062E5}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -4105,7 +4109,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{8ADFB979-1164-474E-A60C-FA148A1D94D6}" type="CELLRANGE">
+                    <a:fld id="{C9183525-29C2-4542-97C0-2BF891FF96A8}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -4144,7 +4148,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{1298A29D-ADD1-7A4E-97B8-3AAAB9C99090}" type="CELLRANGE">
+                    <a:fld id="{EA5C1B6C-5950-914D-AE98-B91797F4B4B4}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -4182,7 +4186,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{9115EC13-5F87-5643-B6CF-E650AD25812E}" type="CELLRANGE">
+                    <a:fld id="{01EEC183-D687-F544-814B-56928A4C2A2B}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -4214,7 +4218,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{14117CDE-C163-2444-950E-117725D65D9B}" type="CELLRANGE">
+                    <a:fld id="{2A2B9F8B-DF5B-9D4C-B38B-22B1741B7721}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -4253,7 +4257,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{6A788B7D-AF83-3E44-84C7-206637D9B99B}" type="CELLRANGE">
+                    <a:fld id="{B60BCF71-8F96-F745-AEDB-270AA1A16207}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -4776,6 +4780,1087 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Correlation</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" baseline="0"/>
+              <a:t> Graph</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t> </a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:dLbl>
+              <c:idx val="0"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-2.7836775668466193E-2"/>
+                  <c:y val="-7.062063115937954E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{56A4A59D-6B14-6548-B883-500C4E208023}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[CELLRANGE]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="en-US"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{0000000F-33EA-B24F-B489-011B761C16D6}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="1"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-2.7836775668466193E-2"/>
+                  <c:y val="9.4160841545839272E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{EC699DE4-9EBA-564E-8C24-A3AB877FB46F}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[CELLRANGE]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="en-US"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000010-33EA-B24F-B489-011B761C16D6}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="2"/>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{DB1A9421-1517-AE41-8583-F23D9C462968}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[CELLRANGE]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="en-US"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000011-33EA-B24F-B489-011B761C16D6}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="3"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-6.4024584037472354E-2"/>
+                  <c:y val="-7.062063115937954E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{84E969E0-BE6A-8948-9E91-0BA70BB3CD0D}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[CELLRANGE]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="en-US"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000012-33EA-B24F-B489-011B761C16D6}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="4"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="7.7942971871705347E-2"/>
+                  <c:y val="-8.9452799468547339E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{4341F845-FEB9-3F4C-B1F9-619D1F648AD6}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[CELLRANGE]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="en-US"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000013-33EA-B24F-B489-011B761C16D6}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="5"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-0.16423697644395055"/>
+                  <c:y val="-0.14124126231875894"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{04EBCA9B-ECF3-0541-A56D-481D9F0D2508}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[CELLRANGE]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="en-US"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000014-33EA-B24F-B489-011B761C16D6}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="6"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-2.2269420534772957E-2"/>
+                  <c:y val="-6.5912589082087511E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{4C94A4FE-FCFA-054C-BFAD-F3D5FD53D645}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[CELLRANGE]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="en-US"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{0000000E-33EA-B24F-B489-011B761C16D6}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="7"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="8.351032700539756E-3"/>
+                  <c:y val="5.1788462850211603E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{FF3893CD-214F-5743-ABDF-452986908D8F}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[CELLRANGE]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="en-US"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000015-33EA-B24F-B489-011B761C16D6}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="8"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-6.1240906470625626E-2"/>
+                  <c:y val="8.0036715313963475E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{089E3CB9-D416-D74C-924C-B050D0A6AC48}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[CELLRANGE]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="en-US"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000016-33EA-B24F-B489-011B761C16D6}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="9"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-0.10577974754017154"/>
+                  <c:y val="-5.6496504927503612E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{E107F226-684D-FD41-99E2-B3F74E2F52B8}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[CELLRANGE]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="en-US"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000017-33EA-B24F-B489-011B761C16D6}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="10"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-0.15310226617656411"/>
+                  <c:y val="-5.1788462850211603E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{6D49CD41-1CE0-5541-84C4-62559571E596}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[CELLRANGE]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="en-US"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000018-33EA-B24F-B489-011B761C16D6}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="11"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-0.11134710267386477"/>
+                  <c:y val="8.4744757391255351E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{307F03C6-E80C-8A4C-B643-8C33918A396F}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[CELLRANGE]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="en-US"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000019-33EA-B24F-B489-011B761C16D6}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:spPr>
+              <a:solidFill>
+                <a:sysClr val="window" lastClr="FFFFFF"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000">
+                    <a:lumMod val="25000"/>
+                    <a:lumOff val="75000"/>
+                  </a:sysClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="dk1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:spPr xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                  <a:prstGeom prst="wedgeRectCallout">
+                    <a:avLst/>
+                  </a:prstGeom>
+                  <a:noFill/>
+                  <a:ln>
+                    <a:noFill/>
+                  </a:ln>
+                </c15:spPr>
+                <c15:showDataLabelsRange val="1"/>
+                <c15:showLeaderLines val="0"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="1"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-0.4259526681727458"/>
+                  <c:y val="-0.36345435987168273"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Corrected SMILES'!$H$2:$H$13</c:f>
+              <c:numCache>
+                <c:formatCode>0.0000</c:formatCode>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>2.8571428600000002</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2.7678571399999998</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2.7555555599999999</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2.6666666700000001</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2.6271186399999999</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2.57261411</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2.57261411</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>2.53061224</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>2.4652087499999999</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>2.4505928899999998</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>2.4077669899999998</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>2.3134328399999999</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Corrected SMILES'!$I$2:$I$13</c:f>
+              <c:numCache>
+                <c:formatCode>0.0000</c:formatCode>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>2.0436926824640902</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2.43509123429157</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.9425545635885999</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2.0714159345870899</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2.4648967372768298</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2.4570679195940102</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2.5192656054505198</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>2.3971570432177001</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>2.1618228925858598</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>2.4330710478370698</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>2.2895097378400302</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>2.23749423811477</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+              <c15:datalabelsRange>
+                <c15:f>'Corrected SMILES'!$G$2:$G$13</c15:f>
+                <c15:dlblRangeCache>
+                  <c:ptCount val="12"/>
+                  <c:pt idx="0">
+                    <c:v>EGUFIZ</c:v>
+                  </c:pt>
+                  <c:pt idx="1">
+                    <c:v>UYOKUR</c:v>
+                  </c:pt>
+                  <c:pt idx="2">
+                    <c:v>EGUFEV</c:v>
+                  </c:pt>
+                  <c:pt idx="3">
+                    <c:v>QAYNOX</c:v>
+                  </c:pt>
+                  <c:pt idx="4">
+                    <c:v>UVEFIM</c:v>
+                  </c:pt>
+                  <c:pt idx="5">
+                    <c:v>CUYRAS</c:v>
+                  </c:pt>
+                  <c:pt idx="6">
+                    <c:v>ATONAB     </c:v>
+                  </c:pt>
+                  <c:pt idx="7">
+                    <c:v>ELOZAI</c:v>
+                  </c:pt>
+                  <c:pt idx="8">
+                    <c:v>ELOYIP</c:v>
+                  </c:pt>
+                  <c:pt idx="9">
+                    <c:v>SOYNOM</c:v>
+                  </c:pt>
+                  <c:pt idx="10">
+                    <c:v>SOYNIG</c:v>
+                  </c:pt>
+                  <c:pt idx="11">
+                    <c:v>UVEFAE</c:v>
+                  </c:pt>
+                </c15:dlblRangeCache>
+              </c15:datalabelsRange>
+            </c:ext>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-33EA-B24F-B489-011B761C16D6}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="748913600"/>
+        <c:axId val="748777392"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="748913600"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:min val="2"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Actual EE</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="0.0000" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="748777392"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="748777392"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:min val="2"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Predicted EE</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="0.0000" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="748913600"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -4817,6 +5902,46 @@
 </file>
 
 <file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -5888,6 +7013,522 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
@@ -5950,6 +7591,47 @@
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{86D8DF25-4F7A-D6DE-2103-96EAF2D0BA11}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>6430</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>10160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>10159</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="6" name="Chart 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{95A3950A-431A-C2E7-CCFA-30D8224100B5}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -8013,7 +9695,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28B6411A-8685-EA48-9958-6ACCD2101161}">
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9.5" bestFit="1" customWidth="1"/>
@@ -8022,7 +9704,7 @@
     <col min="4" max="4" width="23" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -8035,210 +9717,370 @@
       <c r="D1" s="6" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="G1" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="I1" s="6" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>70</v>
       </c>
-      <c r="B2" s="1">
-        <v>2.8770301599999999</v>
-      </c>
+      <c r="B2" s="9">
+        <v>2.8770301624129901</v>
+      </c>
+      <c r="C2" s="9"/>
       <c r="D2" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E2" s="10"/>
+      <c r="G2" t="s">
+        <v>49</v>
+      </c>
+      <c r="H2" s="10">
+        <v>2.8571428600000002</v>
+      </c>
+      <c r="I2" s="9">
+        <v>2.0436926824640902</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>49</v>
       </c>
-      <c r="B3" s="1">
+      <c r="B3" s="10">
         <v>2.8571428600000002</v>
       </c>
+      <c r="C3" s="9">
+        <v>2.0436926824640902</v>
+      </c>
       <c r="D3" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+        <v>75</v>
+      </c>
+      <c r="G3" t="s">
+        <v>12</v>
+      </c>
+      <c r="H3" s="10">
+        <v>2.7678571399999998</v>
+      </c>
+      <c r="I3" s="9">
+        <v>2.43509123429157</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="1">
+      <c r="B4" s="10">
         <v>2.7678571399999998</v>
       </c>
+      <c r="C4" s="9">
+        <v>2.43509123429157</v>
+      </c>
       <c r="D4" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+        <v>75</v>
+      </c>
+      <c r="G4" t="s">
+        <v>48</v>
+      </c>
+      <c r="H4" s="10">
+        <v>2.7555555599999999</v>
+      </c>
+      <c r="I4" s="9">
+        <v>1.9425545635885999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>48</v>
       </c>
-      <c r="B5" s="1">
+      <c r="B5" s="10">
         <v>2.7555555599999999</v>
       </c>
+      <c r="C5" s="9">
+        <v>1.9425545635885999</v>
+      </c>
       <c r="D5" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+        <v>75</v>
+      </c>
+      <c r="G5" t="s">
+        <v>23</v>
+      </c>
+      <c r="H5" s="10">
+        <v>2.6666666700000001</v>
+      </c>
+      <c r="I5" s="9">
+        <v>2.0714159345870899</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>23</v>
       </c>
-      <c r="B6" s="1">
+      <c r="B6" s="10">
         <v>2.6666666700000001</v>
       </c>
       <c r="C6" s="9">
-        <v>1.81898940354585E-12</v>
+        <v>2.0714159345870899</v>
       </c>
       <c r="D6" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="G6" t="s">
+        <v>34</v>
+      </c>
+      <c r="H6" s="10">
+        <v>2.6271186399999999</v>
+      </c>
+      <c r="I6" s="9">
+        <v>2.4648967372768298</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>79</v>
       </c>
-      <c r="B7" s="1">
-        <v>2.6666666700000001</v>
-      </c>
+      <c r="B7" s="9">
+        <v>2.6666666666666599</v>
+      </c>
+      <c r="C7" s="9"/>
       <c r="D7" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E7" s="10"/>
+      <c r="G7" t="s">
+        <v>42</v>
+      </c>
+      <c r="H7" s="10">
+        <v>2.57261411</v>
+      </c>
+      <c r="I7" s="9">
+        <v>2.4570679195940102</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>34</v>
       </c>
-      <c r="B8" s="1">
+      <c r="B8" s="10">
         <v>2.6271186399999999</v>
       </c>
+      <c r="C8" s="9">
+        <v>2.4648967372768298</v>
+      </c>
       <c r="D8" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+        <v>75</v>
+      </c>
+      <c r="G8" t="s">
+        <v>81</v>
+      </c>
+      <c r="H8" s="10">
+        <v>2.57261411</v>
+      </c>
+      <c r="I8" s="9">
+        <v>2.5192656054505198</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>80</v>
       </c>
-      <c r="B9" s="1">
-        <v>2.62156448</v>
-      </c>
+      <c r="B9" s="9">
+        <v>2.6215644820295898</v>
+      </c>
+      <c r="C9" s="9"/>
       <c r="D9" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E9" s="10"/>
+      <c r="G9" t="s">
+        <v>3</v>
+      </c>
+      <c r="H9" s="10">
+        <v>2.53061224</v>
+      </c>
+      <c r="I9" s="9">
+        <v>2.3971570432177001</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>42</v>
       </c>
-      <c r="B10" s="1">
+      <c r="B10" s="10">
         <v>2.57261411</v>
       </c>
       <c r="C10" s="9">
-        <v>9.0949470177292804E-13</v>
+        <v>2.4570679195940102</v>
       </c>
       <c r="D10" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="G10" t="s">
+        <v>6</v>
+      </c>
+      <c r="H10" s="10">
+        <v>2.4652087499999999</v>
+      </c>
+      <c r="I10" s="9">
+        <v>2.1618228925858598</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>81</v>
       </c>
-      <c r="B11" s="1">
+      <c r="B11" s="10">
         <v>2.57261411</v>
       </c>
+      <c r="C11" s="9">
+        <v>2.5192656054505198</v>
+      </c>
       <c r="D11" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+        <v>75</v>
+      </c>
+      <c r="G11" t="s">
+        <v>14</v>
+      </c>
+      <c r="H11" s="10">
+        <v>2.4505928899999998</v>
+      </c>
+      <c r="I11" s="9">
+        <v>2.4330710478370698</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>3</v>
       </c>
-      <c r="B12" s="1">
+      <c r="B12" s="10">
         <v>2.53061224</v>
       </c>
+      <c r="C12" s="9">
+        <v>2.3971570432177001</v>
+      </c>
       <c r="D12" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+        <v>75</v>
+      </c>
+      <c r="G12" t="s">
+        <v>17</v>
+      </c>
+      <c r="H12" s="10">
+        <v>2.4077669899999998</v>
+      </c>
+      <c r="I12" s="9">
+        <v>2.2895097378400302</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>6</v>
       </c>
-      <c r="B13" s="1">
+      <c r="B13" s="10">
         <v>2.4652087499999999</v>
       </c>
+      <c r="C13" s="9">
+        <v>2.1618228925858598</v>
+      </c>
       <c r="D13" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+        <v>75</v>
+      </c>
+      <c r="G13" t="s">
+        <v>35</v>
+      </c>
+      <c r="H13" s="10">
+        <v>2.3134328399999999</v>
+      </c>
+      <c r="I13" s="9">
+        <v>2.23749423811477</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>14</v>
       </c>
-      <c r="B14" s="1">
+      <c r="B14" s="10">
         <v>2.4505928899999998</v>
       </c>
+      <c r="C14" s="9">
+        <v>2.4330710478370698</v>
+      </c>
       <c r="D14" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>17</v>
       </c>
-      <c r="B15" s="1">
+      <c r="B15" s="10">
         <v>2.4077669899999998</v>
       </c>
+      <c r="C15" s="9">
+        <v>2.2895097378400302</v>
+      </c>
       <c r="D15" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>77</v>
       </c>
-      <c r="B16" s="1">
-        <v>2.3529411800000002</v>
-      </c>
+      <c r="B16" s="9">
+        <v>2.3529411764705799</v>
+      </c>
+      <c r="C16" s="9"/>
       <c r="D16" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E16" s="10"/>
+      <c r="I16" s="9"/>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>25</v>
       </c>
-      <c r="B17" s="1">
-        <v>2.33521657</v>
-      </c>
+      <c r="B17" s="9">
+        <v>2.3352165725047</v>
+      </c>
+      <c r="C17" s="9"/>
       <c r="D17" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E17" s="10"/>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>35</v>
       </c>
-      <c r="B18" s="1">
+      <c r="B18" s="10">
         <v>2.3134328399999999</v>
       </c>
+      <c r="C18" s="9">
+        <v>2.23749423811477</v>
+      </c>
       <c r="D18" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>65</v>
       </c>
-      <c r="B19" s="1">
-        <v>2.0981387499999999</v>
-      </c>
+      <c r="B19" s="9">
+        <v>2.0981387478849398</v>
+      </c>
+      <c r="C19" s="9"/>
       <c r="D19" t="s">
         <v>74</v>
       </c>
+      <c r="E19" s="10"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="D1:D19 B20:B1048576">
@@ -8253,5 +10095,6 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>